<commit_message>
Codigo completo con exergo
</commit_message>
<xml_diff>
--- a/Salidas.xlsx
+++ b/Salidas.xlsx
@@ -1,42 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acih0\Documents\CODIGO\tesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{696BD113-F08B-433B-BCFC-F1438E51495D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25F4501-37D5-40F4-BAAB-3B9377582E80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" activeTab="2" xr2:uid="{C4CE93A3-0861-4D2C-B953-37868A8DFB1C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{C4CE93A3-0861-4D2C-B953-37868A8DFB1C}"/>
   </bookViews>
   <sheets>
     <sheet name="T" sheetId="3" r:id="rId1"/>
     <sheet name="Energy_Exergy" sheetId="2" r:id="rId2"/>
-    <sheet name="EXERGO" sheetId="4" r:id="rId3"/>
+    <sheet name="Exergoeconomico" sheetId="5" r:id="rId3"/>
+    <sheet name="EXERGO" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="243">
   <si>
     <t>T [°C]</t>
   </si>
@@ -642,6 +635,129 @@
   </si>
   <si>
     <t>24 ecuaciones</t>
+  </si>
+  <si>
+    <t>Cdot (USD/h)</t>
+  </si>
+  <si>
+    <t>c1</t>
+  </si>
+  <si>
+    <t>c2</t>
+  </si>
+  <si>
+    <t>c3</t>
+  </si>
+  <si>
+    <t>c4</t>
+  </si>
+  <si>
+    <t>c5</t>
+  </si>
+  <si>
+    <t>c6</t>
+  </si>
+  <si>
+    <t>c7</t>
+  </si>
+  <si>
+    <t>c8</t>
+  </si>
+  <si>
+    <t>c9</t>
+  </si>
+  <si>
+    <t>c10</t>
+  </si>
+  <si>
+    <t>c11</t>
+  </si>
+  <si>
+    <t>c12</t>
+  </si>
+  <si>
+    <t>c6BI</t>
+  </si>
+  <si>
+    <t>c6AI</t>
+  </si>
+  <si>
+    <t>c6AO3</t>
+  </si>
+  <si>
+    <t>c6AO</t>
+  </si>
+  <si>
+    <t>c20</t>
+  </si>
+  <si>
+    <t>c15</t>
+  </si>
+  <si>
+    <t>c16</t>
+  </si>
+  <si>
+    <t>c17</t>
+  </si>
+  <si>
+    <t>c18</t>
+  </si>
+  <si>
+    <t>cH2</t>
+  </si>
+  <si>
+    <t>cO2</t>
+  </si>
+  <si>
+    <t>cel</t>
+  </si>
+  <si>
+    <t>Componente</t>
+  </si>
+  <si>
+    <t>c19</t>
+  </si>
+  <si>
+    <t>Evaporador ORC</t>
+  </si>
+  <si>
+    <t>Turbina ORC</t>
+  </si>
+  <si>
+    <t>Bomba ORC</t>
+  </si>
+  <si>
+    <t>Condensador ORC</t>
+  </si>
+  <si>
+    <t>HE-PEM</t>
+  </si>
+  <si>
+    <t>Punto</t>
+  </si>
+  <si>
+    <t>Costo Unit. (USD/kWhex)</t>
+  </si>
+  <si>
+    <t>Zdot (USD/h)</t>
+  </si>
+  <si>
+    <t>ED (kW)</t>
+  </si>
+  <si>
+    <t>CD (USD/h)</t>
+  </si>
+  <si>
+    <t>f (%)</t>
+  </si>
+  <si>
+    <t>LCOEn(USD/kWh)</t>
+  </si>
+  <si>
+    <t>cH2 [USD/kWhex]</t>
+  </si>
+  <si>
+    <t>cElectricidad [USD/kWhex]</t>
   </si>
 </sst>
 </file>
@@ -753,7 +869,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -812,6 +928,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -880,9 +998,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -920,7 +1038,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1026,7 +1144,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1168,7 +1286,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1266,34 +1384,34 @@
         <v>500</v>
       </c>
       <c r="C3" s="19">
-        <v>0.79959526453496776</v>
+        <v>7.9817560813786423</v>
       </c>
       <c r="D3" s="17">
-        <v>5.7474602609853757E-2</v>
+        <v>0.57478365564259748</v>
       </c>
       <c r="E3" s="19">
-        <v>44.242025146810107</v>
+        <v>44.197489238670407</v>
       </c>
       <c r="F3" s="19">
-        <v>22.280941712184308</v>
+        <v>22.006324234413263</v>
       </c>
       <c r="G3" s="19">
-        <v>42.805350727912341</v>
+        <v>42.266069418369199</v>
       </c>
       <c r="H3" s="19">
-        <v>54.391713608301288</v>
+        <v>39.083036578748462</v>
       </c>
       <c r="I3" s="19">
-        <v>53.43053490915559</v>
+        <v>38.322157470640676</v>
       </c>
       <c r="J3" s="19">
-        <v>71.431846289059933</v>
+        <v>73.705196115616388</v>
       </c>
       <c r="K3" s="19">
-        <v>0.94449159071981759</v>
+        <v>6.7738392475312912</v>
       </c>
       <c r="L3" s="17">
-        <v>8.4406216959654934</v>
+        <v>60.535652280525397</v>
       </c>
       <c r="M3" s="21"/>
       <c r="N3" s="21"/>
@@ -1323,34 +1441,34 @@
         <v>550</v>
       </c>
       <c r="C4" s="17">
-        <v>0.89972160669047219</v>
+        <v>8.9819868548594588</v>
       </c>
       <c r="D4" s="17">
-        <v>5.9775959042112747E-2</v>
+        <v>0.59780007016897552</v>
       </c>
       <c r="E4" s="17">
-        <v>46.738186634220291</v>
+        <v>46.69526627123269</v>
       </c>
       <c r="F4" s="17">
-        <v>23.115653468129583</v>
+        <v>22.850005374764851</v>
       </c>
       <c r="G4" s="17">
-        <v>45.32985739384808</v>
+        <v>44.797301420947292</v>
       </c>
       <c r="H4" s="17">
-        <v>54.219471799935384</v>
+        <v>38.702038861674041</v>
       </c>
       <c r="I4" s="17">
-        <v>53.258556160364932</v>
+        <v>37.945565695998773</v>
       </c>
       <c r="J4" s="17">
-        <v>71.235617634821836</v>
+        <v>73.460227385209635</v>
       </c>
       <c r="K4" s="17">
-        <v>0.97914227476891347</v>
+        <v>6.9757969550625445</v>
       </c>
       <c r="L4" s="17">
-        <v>8.7502838660033913</v>
+        <v>62.340484239438453</v>
       </c>
       <c r="M4" s="21"/>
       <c r="N4" s="21"/>
@@ -1380,34 +1498,34 @@
         <v>600</v>
       </c>
       <c r="C5" s="17">
-        <v>0.99841792896138692</v>
+        <v>9.9679334582948602</v>
       </c>
       <c r="D5" s="17">
-        <v>6.2107603556281796E-2</v>
+        <v>0.62111932846844753</v>
       </c>
       <c r="E5" s="17">
-        <v>48.905256206618859</v>
+        <v>48.863771870449504</v>
       </c>
       <c r="F5" s="17">
-        <v>23.650319962765966</v>
+        <v>23.39359126526438</v>
       </c>
       <c r="G5" s="17">
-        <v>47.52015705474146</v>
+        <v>46.992751286845909</v>
       </c>
       <c r="H5" s="17">
-        <v>54.048316611557979</v>
+        <v>38.328127919305047</v>
       </c>
       <c r="I5" s="17">
-        <v>53.087671766748116</v>
+        <v>37.576039107764217</v>
       </c>
       <c r="J5" s="17">
-        <v>71.038424425410881</v>
+        <v>73.215836655735927</v>
       </c>
       <c r="K5" s="17">
-        <v>1.0140645281447851</v>
+        <v>7.1772698736697782</v>
       </c>
       <c r="L5" s="17">
-        <v>9.0623729649563405</v>
+        <v>64.140983793542134</v>
       </c>
       <c r="M5" s="21"/>
       <c r="N5" s="21"/>
@@ -1437,34 +1555,34 @@
         <v>650</v>
       </c>
       <c r="C6" s="17">
-        <v>1.095976970270373</v>
+        <v>10.942520132883478</v>
       </c>
       <c r="D6" s="17">
-        <v>6.4468832600220724E-2</v>
+        <v>0.6447344000410401</v>
       </c>
       <c r="E6" s="17">
-        <v>50.80680659983301</v>
+        <v>50.766607886856718</v>
       </c>
       <c r="F6" s="17">
-        <v>23.908927906115419</v>
+        <v>23.661351320584064</v>
       </c>
       <c r="G6" s="17">
-        <v>49.440886587190505</v>
+        <v>48.91739667752401</v>
       </c>
       <c r="H6" s="17">
-        <v>53.878220178726544</v>
+        <v>37.961182417304968</v>
       </c>
       <c r="I6" s="17">
-        <v>52.917855462200883</v>
+        <v>37.213454717865027</v>
       </c>
       <c r="J6" s="17">
-        <v>70.840471045585389</v>
+        <v>72.972155033057845</v>
       </c>
       <c r="K6" s="17">
-        <v>1.0492439615518117</v>
+        <v>7.3782020252319311</v>
       </c>
       <c r="L6" s="17">
-        <v>9.3767604002545415</v>
+        <v>65.936650684128182</v>
       </c>
       <c r="M6" s="21"/>
       <c r="N6" s="21"/>
@@ -1494,34 +1612,34 @@
         <v>700</v>
       </c>
       <c r="C7" s="17">
-        <v>1.1926154214167359</v>
+        <v>11.907911442755228</v>
       </c>
       <c r="D7" s="17">
-        <v>6.6858338839570361E-2</v>
+        <v>0.66863221481329138</v>
       </c>
       <c r="E7" s="17">
-        <v>52.490240359052798</v>
+        <v>52.451199641588161</v>
       </c>
       <c r="F7" s="17">
-        <v>23.905414304807127</v>
+        <v>23.667463179486298</v>
       </c>
       <c r="G7" s="17">
-        <v>51.140240176954421</v>
+        <v>50.619687111767362</v>
       </c>
       <c r="H7" s="17">
-        <v>53.709201785475713</v>
+        <v>37.60117137295029</v>
       </c>
       <c r="I7" s="17">
-        <v>52.749127913968607</v>
+        <v>36.857778908474963</v>
       </c>
       <c r="J7" s="17">
-        <v>70.642003533187847</v>
+        <v>72.729372195994642</v>
       </c>
       <c r="K7" s="17">
-        <v>1.08465748785521</v>
+        <v>7.5784907719207091</v>
       </c>
       <c r="L7" s="17">
-        <v>9.6932398494990846</v>
+        <v>67.726567669488134</v>
       </c>
       <c r="M7" s="21"/>
       <c r="N7" s="21"/>
@@ -1551,34 +1669,34 @@
         <v>750</v>
       </c>
       <c r="C8" s="17">
-        <v>1.2884976984183187</v>
+        <v>12.865749758364128</v>
       </c>
       <c r="D8" s="17">
-        <v>6.9274475184734868E-2</v>
+        <v>0.6927963040732894</v>
       </c>
       <c r="E8" s="17">
-        <v>53.991830167895671</v>
+        <v>53.953838014043107</v>
       </c>
       <c r="F8" s="17">
-        <v>23.646581930865896</v>
+        <v>23.418942554906867</v>
       </c>
       <c r="G8" s="17">
-        <v>52.655094193700535</v>
+        <v>52.136694846180184</v>
       </c>
       <c r="H8" s="17">
-        <v>53.541305493071732</v>
+        <v>37.248102901082589</v>
       </c>
       <c r="I8" s="17">
-        <v>52.581534383252716</v>
+        <v>36.50901673542819</v>
       </c>
       <c r="J8" s="17">
-        <v>70.44328600163891</v>
+        <v>72.487705338327999</v>
       </c>
       <c r="K8" s="17">
-        <v>1.1202774409417275</v>
+        <v>7.7780119622835953</v>
       </c>
       <c r="L8" s="17">
-        <v>10.011564069413204</v>
+        <v>69.509625247479235</v>
       </c>
       <c r="M8" s="21"/>
       <c r="N8" s="21"/>
@@ -1608,34 +1726,34 @@
         <v>800.00000000000011</v>
       </c>
       <c r="C9" s="17">
-        <v>1.3837514731671954</v>
+        <v>13.817310399416089</v>
       </c>
       <c r="D9" s="17">
-        <v>7.1715431970801227E-2</v>
+        <v>0.71720857262984272</v>
       </c>
       <c r="E9" s="17">
-        <v>55.339933569630354</v>
+        <v>55.302895315550685</v>
       </c>
       <c r="F9" s="17">
-        <v>23.133959295545651</v>
+        <v>22.917512377362197</v>
       </c>
       <c r="G9" s="17">
-        <v>54.014275766007323</v>
+        <v>53.497400064021491</v>
       </c>
       <c r="H9" s="17">
-        <v>53.374586045417935</v>
+        <v>36.901993581878948</v>
       </c>
       <c r="I9" s="17">
-        <v>52.415130655682205</v>
+        <v>36.167181648495081</v>
       </c>
       <c r="J9" s="17">
-        <v>70.244585496392403</v>
+        <v>72.247379706631875</v>
       </c>
       <c r="K9" s="17">
-        <v>1.1560742978764087</v>
+        <v>7.9766358915200142</v>
       </c>
       <c r="L9" s="17">
-        <v>10.331469222893681</v>
+        <v>71.284664287449004</v>
       </c>
       <c r="M9" s="21"/>
       <c r="N9" s="21"/>
@@ -1839,64 +1957,64 @@
         <v>500</v>
       </c>
       <c r="C16" s="17">
-        <v>29.485120651710428</v>
+        <v>294.85614292537934</v>
       </c>
       <c r="D16" s="17">
-        <v>13.564888381060969</v>
+        <v>135.64262301173875</v>
       </c>
       <c r="E16" s="17">
-        <v>14.906637101063389</v>
+        <v>151.19146157877427</v>
       </c>
       <c r="F16" s="17">
-        <v>27.324224769671563</v>
+        <v>277.13026251072807</v>
       </c>
       <c r="G16" s="17">
-        <v>8.6106797085443318</v>
+        <v>86.111522976340609</v>
       </c>
       <c r="H16" s="17">
-        <v>3.3947199989052024</v>
+        <v>34.017747966403839</v>
       </c>
       <c r="I16" s="17">
-        <v>30.271704873401731</v>
+        <v>302.81716564914211</v>
       </c>
       <c r="J16" s="17">
-        <v>118.03699553521798</v>
+        <v>1179.4615416517445</v>
       </c>
       <c r="K16" s="17">
-        <v>1387.4581203814137</v>
+        <v>13863.903314567468</v>
       </c>
       <c r="L16" s="17">
-        <v>894.0177603515491</v>
+        <v>8932.9858804423748</v>
       </c>
       <c r="M16" s="17">
-        <v>3.2636063061677061</v>
+        <v>3.3626344503154937</v>
       </c>
       <c r="N16" s="17">
-        <v>1.6493762302839108</v>
+        <v>1.6493321533075163</v>
       </c>
       <c r="O16" s="17">
-        <v>66.202538828775772</v>
+        <v>662.01750343054505</v>
       </c>
       <c r="P16" s="17">
-        <v>30.731160961602338</v>
+        <v>307.33893335012613</v>
       </c>
       <c r="Q16" s="17">
-        <v>0</v>
+        <v>6.9940860806835592E-2</v>
       </c>
       <c r="R16" s="17">
-        <v>6.3532146035785448</v>
+        <v>63.537030855789887</v>
       </c>
       <c r="S16" s="17">
-        <v>33.747118549449517</v>
+        <v>381.6564040682814</v>
       </c>
       <c r="T16" s="17">
-        <v>3468.6453009535339</v>
+        <v>34659.75828641867</v>
       </c>
       <c r="U16" s="17">
-        <v>26.639387578646851</v>
+        <v>353.65731761283195</v>
       </c>
       <c r="V16" s="17">
-        <v>2695.657254811043</v>
+        <v>27031.406760062098</v>
       </c>
     </row>
     <row r="17" spans="2:26" x14ac:dyDescent="0.3">
@@ -1904,64 +2022,64 @@
         <v>550</v>
       </c>
       <c r="C17" s="17">
-        <v>29.781783917630268</v>
+        <v>297.82296698241635</v>
       </c>
       <c r="D17" s="17">
-        <v>13.187459854217858</v>
+        <v>131.86805418472457</v>
       </c>
       <c r="E17" s="17">
-        <v>15.005112575197126</v>
+        <v>152.19025287038554</v>
       </c>
       <c r="F17" s="17">
-        <v>27.447206193680177</v>
+        <v>278.37767920301479</v>
       </c>
       <c r="G17" s="17">
-        <v>8.8978395707103122</v>
+        <v>88.983413920749442</v>
       </c>
       <c r="H17" s="17">
-        <v>8.045436130908783</v>
+        <v>80.540884684346381</v>
       </c>
       <c r="I17" s="17">
-        <v>36.484341624139283</v>
+        <v>364.95425807604568</v>
       </c>
       <c r="J17" s="17">
-        <v>159.28762450721621</v>
+        <v>1591.6416778681469</v>
       </c>
       <c r="K17" s="17">
-        <v>1508.5865165479815</v>
+        <v>15074.172785462781</v>
       </c>
       <c r="L17" s="17">
-        <v>917.31651422341099</v>
+        <v>9165.742924421842</v>
       </c>
       <c r="M17" s="17">
-        <v>3.229940708208169</v>
+        <v>3.3261513919689558</v>
       </c>
       <c r="N17" s="17">
-        <v>1.6227368839905512</v>
+        <v>1.6226905804250538</v>
       </c>
       <c r="O17" s="17">
-        <v>70.030539355826804</v>
+        <v>700.30101822417953</v>
       </c>
       <c r="P17" s="17">
-        <v>32.431629299966701</v>
+        <v>324.34672934535394</v>
       </c>
       <c r="Q17" s="17">
-        <v>0</v>
+        <v>7.2279964988682083E-2</v>
       </c>
       <c r="R17" s="17">
-        <v>6.6540307771452101</v>
+        <v>66.545635698113529</v>
       </c>
       <c r="S17" s="17">
-        <v>33.7028919835547</v>
+        <v>380.67789920895763</v>
       </c>
       <c r="T17" s="17">
-        <v>3771.4662913699544</v>
+        <v>37685.431963656949</v>
       </c>
       <c r="U17" s="17">
-        <v>27.809219672175992</v>
+        <v>370.07849924618142</v>
       </c>
       <c r="V17" s="17">
-        <v>2899.5208238259606</v>
+        <v>29073.265801334615</v>
       </c>
     </row>
     <row r="18" spans="2:26" x14ac:dyDescent="0.3">
@@ -1969,64 +2087,64 @@
         <v>600</v>
       </c>
       <c r="C18" s="17">
-        <v>30.072126059584438</v>
+        <v>300.72656005696859</v>
       </c>
       <c r="D18" s="17">
-        <v>12.815757813462639</v>
+        <v>128.15077235300279</v>
       </c>
       <c r="E18" s="17">
-        <v>15.074997029094375</v>
+        <v>152.89907199523319</v>
       </c>
       <c r="F18" s="17">
-        <v>27.53273934130091</v>
+        <v>279.2453075698167</v>
       </c>
       <c r="G18" s="17">
-        <v>9.1850023844852036</v>
+        <v>91.855320754454354</v>
       </c>
       <c r="H18" s="17">
-        <v>13.191794613489183</v>
+        <v>132.01571327555575</v>
       </c>
       <c r="I18" s="17">
-        <v>42.957817343885893</v>
+        <v>429.70000918122383</v>
       </c>
       <c r="J18" s="17">
-        <v>212.54457106783326</v>
+        <v>2123.7887994432162</v>
       </c>
       <c r="K18" s="17">
-        <v>1639.3855942730463</v>
+        <v>16381.075957825688</v>
       </c>
       <c r="L18" s="17">
-        <v>943.66296676565219</v>
+        <v>9428.9610392787527</v>
       </c>
       <c r="M18" s="17">
-        <v>3.1964045904803005</v>
+        <v>3.2898953561125701</v>
       </c>
       <c r="N18" s="17">
-        <v>1.5963807829348928</v>
+        <v>1.5963324264198737</v>
       </c>
       <c r="O18" s="17">
-        <v>73.974395706709728</v>
+        <v>739.74316456090378</v>
       </c>
       <c r="P18" s="17">
-        <v>34.216175837851559</v>
+        <v>342.19548588824279</v>
       </c>
       <c r="Q18" s="17">
-        <v>0</v>
+        <v>7.4619661227411427E-2</v>
       </c>
       <c r="R18" s="17">
-        <v>6.9630843835348282</v>
+        <v>69.636622761948459</v>
       </c>
       <c r="S18" s="17">
-        <v>33.642267122887539</v>
+        <v>379.53905784855749</v>
       </c>
       <c r="T18" s="17">
-        <v>4098.4639856826152</v>
+        <v>40952.68989456421</v>
       </c>
       <c r="U18" s="17">
-        <v>29.00045429948581</v>
+        <v>386.81822347694612</v>
       </c>
       <c r="V18" s="17">
-        <v>3129.0125294157187</v>
+        <v>31371.31195371427</v>
       </c>
     </row>
     <row r="19" spans="2:26" x14ac:dyDescent="0.3">
@@ -2034,64 +2152,64 @@
         <v>650</v>
       </c>
       <c r="C19" s="17">
-        <v>30.356348204785782</v>
+        <v>303.5689357492202</v>
       </c>
       <c r="D19" s="17">
-        <v>12.44961559979507</v>
+        <v>124.48910840925201</v>
       </c>
       <c r="E19" s="17">
-        <v>15.124260333639103</v>
+        <v>153.39874970301798</v>
       </c>
       <c r="F19" s="17">
-        <v>27.591578472916037</v>
+        <v>279.8422102253549</v>
       </c>
       <c r="G19" s="17">
-        <v>9.4719934814589077</v>
+        <v>94.725497642047941</v>
       </c>
       <c r="H19" s="17">
-        <v>18.57419322769216</v>
+        <v>185.84739014316</v>
       </c>
       <c r="I19" s="17">
-        <v>49.691064890158593</v>
+        <v>497.04374229533039</v>
       </c>
       <c r="J19" s="17">
-        <v>281.0885470546134</v>
+        <v>2808.6836717508977</v>
       </c>
       <c r="K19" s="17">
-        <v>1782.8354646964092</v>
+        <v>17814.38949249798</v>
       </c>
       <c r="L19" s="17">
-        <v>974.191411747036</v>
+        <v>9733.9721439540208</v>
       </c>
       <c r="M19" s="17">
-        <v>3.1630198633730169</v>
+        <v>3.2538839114981575</v>
       </c>
       <c r="N19" s="17">
-        <v>1.5703191740388991</v>
+        <v>1.570268926036658</v>
       </c>
       <c r="O19" s="17">
-        <v>78.033235234910777</v>
+        <v>780.3352173446757</v>
       </c>
       <c r="P19" s="17">
-        <v>36.089167156528923</v>
+        <v>360.9288825433681</v>
       </c>
       <c r="Q19" s="17">
-        <v>0</v>
+        <v>7.6958539798279726E-2</v>
       </c>
       <c r="R19" s="17">
-        <v>7.2805324924249097</v>
+        <v>72.811563723715722</v>
       </c>
       <c r="S19" s="17">
-        <v>33.566067839114389</v>
+        <v>378.24841917647922</v>
       </c>
       <c r="T19" s="17">
-        <v>4457.0886617410233</v>
+        <v>44535.973731244943</v>
       </c>
       <c r="U19" s="17">
-        <v>30.212857749627148</v>
+        <v>403.8712905190423</v>
       </c>
       <c r="V19" s="17">
-        <v>3391.2896772185222</v>
+        <v>33997.057427054897</v>
       </c>
     </row>
     <row r="20" spans="2:26" x14ac:dyDescent="0.3">
@@ -2099,64 +2217,64 @@
         <v>700</v>
       </c>
       <c r="C20" s="17">
-        <v>30.634572596853715</v>
+        <v>306.35131841675008</v>
       </c>
       <c r="D20" s="17">
-        <v>12.088966631737916</v>
+        <v>120.88239449501667</v>
       </c>
       <c r="E20" s="17">
-        <v>15.158362934418255</v>
+        <v>153.74467368248199</v>
       </c>
       <c r="F20" s="17">
-        <v>27.631189878644655</v>
+        <v>280.24408784225767</v>
       </c>
       <c r="G20" s="17">
-        <v>9.7585717022123273</v>
+        <v>97.59153362218035</v>
       </c>
       <c r="H20" s="17">
-        <v>24.020430877263426</v>
+        <v>240.31475528596201</v>
       </c>
       <c r="I20" s="17">
-        <v>56.681040389213244</v>
+        <v>566.95500958230537</v>
       </c>
       <c r="J20" s="17">
-        <v>369.23294106569756</v>
+        <v>3689.4255484164842</v>
       </c>
       <c r="K20" s="17">
-        <v>1942.7283156258552</v>
+        <v>19412.004412755879</v>
       </c>
       <c r="L20" s="17">
-        <v>1010.2197197239223</v>
+        <v>10093.94296158151</v>
       </c>
       <c r="M20" s="17">
-        <v>3.1298159081650674</v>
+        <v>3.2181430517416656</v>
       </c>
       <c r="N20" s="17">
-        <v>1.5445691713135157</v>
+        <v>1.544517183389571</v>
       </c>
       <c r="O20" s="17">
-        <v>82.204971307235269</v>
+        <v>822.05630927133234</v>
       </c>
       <c r="P20" s="17">
-        <v>38.054574357161769</v>
+        <v>380.58664247568697</v>
       </c>
       <c r="Q20" s="17">
-        <v>0</v>
+        <v>7.9294647204591173E-2</v>
       </c>
       <c r="R20" s="17">
-        <v>7.6064535049367379</v>
+        <v>76.071243546232026</v>
       </c>
       <c r="S20" s="17">
-        <v>33.475120850675864</v>
+        <v>376.81466876953999</v>
       </c>
       <c r="T20" s="17">
-        <v>4856.8207890646372</v>
+        <v>48530.011031889699</v>
       </c>
       <c r="U20" s="17">
-        <v>31.445876616620488</v>
+        <v>421.22798507395089</v>
       </c>
       <c r="V20" s="17">
-        <v>3695.6154931419278</v>
+        <v>37043.055499699934</v>
       </c>
     </row>
     <row r="21" spans="2:26" x14ac:dyDescent="0.3">
@@ -2164,64 +2282,64 @@
         <v>750</v>
       </c>
       <c r="C21" s="17">
-        <v>30.906883731184411</v>
+        <v>309.07455465127805</v>
       </c>
       <c r="D21" s="17">
-        <v>11.733793427656783</v>
+        <v>117.33045407099952</v>
       </c>
       <c r="E21" s="17">
-        <v>15.181449948766968</v>
+        <v>153.97884766306913</v>
       </c>
       <c r="F21" s="17">
-        <v>27.656590211398434</v>
+        <v>280.50183820071442</v>
       </c>
       <c r="G21" s="17">
-        <v>10.044465293963134</v>
+        <v>100.45071167206741</v>
       </c>
       <c r="H21" s="17">
-        <v>29.414976429465458</v>
+        <v>294.26310690947577</v>
       </c>
       <c r="I21" s="17">
-        <v>63.923314061612821</v>
+        <v>639.38950186234808</v>
       </c>
       <c r="J21" s="17">
-        <v>482.7644158839729</v>
+        <v>4823.8346125543394</v>
       </c>
       <c r="K21" s="17">
-        <v>2124.0584594927946</v>
+        <v>21223.823419605003</v>
       </c>
       <c r="L21" s="17">
-        <v>1053.3975711688122</v>
+        <v>10525.356004225263</v>
       </c>
       <c r="M21" s="17">
-        <v>3.096825295401116</v>
+        <v>3.182702476477075</v>
       </c>
       <c r="N21" s="17">
-        <v>1.5191502375896373</v>
+        <v>1.519096652861311</v>
       </c>
       <c r="O21" s="17">
-        <v>86.486698692361983</v>
+        <v>864.87738547050515</v>
       </c>
       <c r="P21" s="17">
-        <v>40.11610028928925</v>
+        <v>401.20580558999745</v>
       </c>
       <c r="Q21" s="17">
-        <v>0</v>
+        <v>8.1625778220241155E-2</v>
       </c>
       <c r="R21" s="17">
-        <v>7.940877684283616</v>
+        <v>79.415965355949552</v>
       </c>
       <c r="S21" s="17">
-        <v>33.370260142907128</v>
+        <v>375.24661356442857</v>
       </c>
       <c r="T21" s="17">
-        <v>5310.1461487319866</v>
+        <v>53059.558549012494</v>
       </c>
       <c r="U21" s="17">
-        <v>32.698767335133454</v>
+        <v>438.8758961478494</v>
       </c>
       <c r="V21" s="17">
-        <v>4054.3105993265945</v>
+        <v>40632.408142450848</v>
       </c>
     </row>
     <row r="22" spans="2:26" x14ac:dyDescent="0.3">
@@ -2229,64 +2347,64 @@
         <v>800.00000000000011</v>
       </c>
       <c r="C22" s="17">
-        <v>31.17335186523071</v>
+        <v>311.73934843303778</v>
       </c>
       <c r="D22" s="17">
-        <v>11.384097947699106</v>
+        <v>113.83330527634081</v>
       </c>
       <c r="E22" s="17">
-        <v>15.196049134857022</v>
+        <v>154.12694860114715</v>
       </c>
       <c r="F22" s="17">
-        <v>27.671506806551477</v>
+        <v>280.65325482354871</v>
       </c>
       <c r="G22" s="17">
-        <v>10.329389197445023</v>
+        <v>103.30018156282743</v>
       </c>
       <c r="H22" s="17">
-        <v>34.679829083029183</v>
+        <v>346.91288051130834</v>
       </c>
       <c r="I22" s="17">
-        <v>71.412496173838846</v>
+        <v>714.29330882120883</v>
       </c>
       <c r="J22" s="17">
-        <v>629.63432798074223</v>
+        <v>6291.3606293226931</v>
       </c>
       <c r="K22" s="17">
-        <v>2333.6176965557079</v>
+        <v>23317.709736516052</v>
       </c>
       <c r="L22" s="17">
-        <v>1105.9100285509264</v>
+        <v>11050.043569183621</v>
       </c>
       <c r="M22" s="17">
-        <v>3.0640811169153399</v>
+        <v>3.1475926729674328</v>
       </c>
       <c r="N22" s="17">
-        <v>1.4940820414417189</v>
+        <v>1.4940269956205496</v>
       </c>
       <c r="O22" s="17">
-        <v>90.874967050593952</v>
+        <v>908.7639387171597</v>
       </c>
       <c r="P22" s="17">
-        <v>42.277260541399329</v>
+        <v>422.82153795985045</v>
       </c>
       <c r="Q22" s="17">
-        <v>0</v>
+        <v>8.3949658717157039E-2</v>
       </c>
       <c r="R22" s="17">
-        <v>8.2838071011636547</v>
+        <v>82.84575052116061</v>
       </c>
       <c r="S22" s="17">
-        <v>33.252324097050263</v>
+        <v>373.5531104491323</v>
       </c>
       <c r="T22" s="17">
-        <v>5834.0442413892697</v>
+        <v>58294.274341290125</v>
       </c>
       <c r="U22" s="17">
-        <v>33.970684470386352</v>
+        <v>456.8011680060402</v>
       </c>
       <c r="V22" s="17">
-        <v>4484.2259797149791</v>
+        <v>44933.484238032433</v>
       </c>
       <c r="W22" s="21"/>
       <c r="X22" s="21"/>
@@ -2365,22 +2483,22 @@
         <v>500</v>
       </c>
       <c r="C29" s="17">
-        <v>0.77714987291148052</v>
+        <v>0.77990753820849013</v>
       </c>
       <c r="D29" s="17">
-        <v>3.4879579281269653</v>
+        <v>3.5440154834621529</v>
       </c>
       <c r="E29" s="21">
-        <v>0.28670070585885776</v>
+        <v>0.28216581012876918</v>
       </c>
       <c r="F29" s="21">
-        <v>1.1542250716925242E-2</v>
+        <v>1.1512137739935889E-2</v>
       </c>
       <c r="G29">
-        <v>0.67842275179467249</v>
+        <v>0.67677225952588616</v>
       </c>
       <c r="H29">
-        <v>22.285012708851948</v>
+        <v>22.009246179150999</v>
       </c>
       <c r="I29" s="25"/>
       <c r="J29" s="25"/>
@@ -2390,22 +2508,22 @@
         <v>550</v>
       </c>
       <c r="C30" s="17">
-        <v>0.76880465045141189</v>
+        <v>0.77147227154971376</v>
       </c>
       <c r="D30" s="17">
-        <v>3.3259048960540598</v>
+        <v>3.3762454708291418</v>
       </c>
       <c r="E30" s="21">
-        <v>0.30067005258822227</v>
+        <v>0.29618699488530348</v>
       </c>
       <c r="F30" s="21">
-        <v>1.147679867865287E-2</v>
+        <v>1.1448741730107946E-2</v>
       </c>
       <c r="G30">
-        <v>0.6748353255769638</v>
+        <v>0.67329752422721656</v>
       </c>
       <c r="H30">
-        <v>23.11953495485881</v>
+        <v>22.852772845028625</v>
       </c>
       <c r="I30" s="25"/>
       <c r="J30" s="25"/>
@@ -2415,22 +2533,22 @@
         <v>600</v>
       </c>
       <c r="C31" s="17">
-        <v>0.76345980844200811</v>
+        <v>0.76603788504447645</v>
       </c>
       <c r="D31" s="17">
-        <v>3.2281161931169047</v>
+        <v>3.2745630047059779</v>
       </c>
       <c r="E31" s="21">
-        <v>0.30977819265992745</v>
+        <v>0.30538425999526303</v>
       </c>
       <c r="F31" s="21">
-        <v>1.1426248092306848E-2</v>
+        <v>1.1402542302703553E-2</v>
       </c>
       <c r="G31">
-        <v>0.6720646479393384</v>
+        <v>0.67076533361118174</v>
       </c>
       <c r="H31">
-        <v>23.654019155799176</v>
+        <v>23.396211495552354</v>
       </c>
       <c r="I31" s="25"/>
       <c r="J31" s="25"/>
@@ -2440,22 +2558,22 @@
         <v>650</v>
       </c>
       <c r="C32" s="17">
-        <v>0.76087552539146053</v>
+        <v>0.76336171815198695</v>
       </c>
       <c r="D32" s="17">
-        <v>3.1823908139220412</v>
+        <v>3.2261966267662174</v>
       </c>
       <c r="E32" s="21">
-        <v>0.31422916243513799</v>
+        <v>0.30996250870250008</v>
       </c>
       <c r="F32" s="21">
-        <v>1.1389377536649816E-2</v>
+        <v>1.1366515645355346E-2</v>
       </c>
       <c r="G32">
-        <v>0.67004377278377647</v>
+        <v>0.66879071252192657</v>
       </c>
       <c r="H32">
-        <v>23.912447460853958</v>
+        <v>23.663828184801304</v>
       </c>
       <c r="I32" s="25"/>
       <c r="J32" s="25"/>
@@ -2465,22 +2583,22 @@
         <v>700</v>
       </c>
       <c r="C33" s="17">
-        <v>0.76091246797962597</v>
+        <v>0.76330202099806788</v>
       </c>
       <c r="D33" s="17">
-        <v>3.1830130960190659</v>
+        <v>3.2251112643946462</v>
       </c>
       <c r="E33" s="21">
-        <v>0.31416773033409162</v>
+        <v>0.31006682189232937</v>
       </c>
       <c r="F33" s="21">
-        <v>1.1358039352888392E-2</v>
+        <v>1.1337655298378537E-2</v>
       </c>
       <c r="G33">
-        <v>0.66832612693181281</v>
+        <v>0.66720887690412767</v>
       </c>
       <c r="H33">
-        <v>23.908753202037392</v>
+        <v>23.669797900193213</v>
       </c>
       <c r="I33" s="25"/>
       <c r="J33" s="25"/>
@@ -2490,22 +2608,22 @@
         <v>750</v>
       </c>
       <c r="C34" s="17">
-        <v>0.76350263924369122</v>
+        <v>0.76578865813437991</v>
       </c>
       <c r="D34" s="17">
-        <v>3.2288076199591909</v>
+        <v>3.269954039722121</v>
       </c>
       <c r="E34" s="21">
-        <v>0.30971185580038957</v>
+        <v>0.30581469581908238</v>
       </c>
       <c r="F34" s="21">
-        <v>1.1333787980593049E-2</v>
+        <v>1.1313771415970319E-2</v>
       </c>
       <c r="G34">
-        <v>0.66699690921630506</v>
+        <v>0.66589980130933324</v>
       </c>
       <c r="H34">
-        <v>23.649736075630877</v>
+        <v>23.421134186562</v>
       </c>
       <c r="I34" s="25"/>
       <c r="J34" s="25"/>
@@ -2515,22 +2633,22 @@
         <v>800.00000000000011</v>
       </c>
       <c r="C35" s="17">
-        <v>0.76863078066873625</v>
+        <v>0.77080441854314019</v>
       </c>
       <c r="D35" s="17">
-        <v>3.3225215400838581</v>
+        <v>3.3633860684833179</v>
       </c>
       <c r="E35" s="21">
-        <v>0.30097622782447353</v>
+        <v>0.29731942145165008</v>
       </c>
       <c r="F35" s="21">
-        <v>1.131159921198268E-2</v>
+        <v>1.1293500510283605E-2</v>
       </c>
       <c r="G35">
-        <v>0.66578074280877075</v>
+        <v>0.66478875296864437</v>
       </c>
       <c r="H35">
-        <v>23.136921933126388</v>
+        <v>22.919558145685983</v>
       </c>
       <c r="I35" s="25"/>
       <c r="J35" s="25"/>
@@ -2575,7 +2693,7 @@
     <col min="17" max="17" width="24.109375" customWidth="1"/>
     <col min="18" max="18" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="14.6640625" customWidth="1"/>
-    <col min="20" max="20" width="13.21875" customWidth="1"/>
+    <col min="20" max="20" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.3">
@@ -2633,7 +2751,7 @@
         <v>3.0305681085599816</v>
       </c>
       <c r="G3" s="4">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="H3" s="4">
         <v>756.61237274082237</v>
@@ -2666,44 +2784,44 @@
         <v>2</v>
       </c>
       <c r="C4" s="4">
-        <v>1018.1289616795918</v>
+        <v>1018.1871360117831</v>
       </c>
       <c r="D4" s="5">
         <v>17.482517482517483</v>
       </c>
       <c r="E4" s="4">
-        <v>1281.2341664776559</v>
+        <v>1281.3081492359206</v>
       </c>
       <c r="F4" s="7">
-        <v>3.035664888414034</v>
+        <v>3.0357375517463359</v>
       </c>
       <c r="G4" s="4">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="H4" s="4">
-        <v>686.28880264133011</v>
+        <v>686.34112082706883</v>
       </c>
       <c r="I4" s="4">
         <f t="shared" ref="I4:I42" si="0">C4-273.15</f>
-        <v>744.97896167959186</v>
+        <v>745.0371360117831</v>
       </c>
       <c r="K4" s="9" t="s">
         <v>42</v>
       </c>
       <c r="L4" s="7">
-        <v>1.7979758880009502</v>
+        <v>17.967369630276828</v>
       </c>
       <c r="N4" s="9" t="s">
         <v>66</v>
       </c>
       <c r="O4" s="10">
-        <v>688.03965186006621</v>
+        <v>6872.9982427742098</v>
       </c>
       <c r="Q4" s="13" t="s">
         <v>98</v>
       </c>
       <c r="R4" s="6">
-        <v>916.98727526679568</v>
+        <v>3089.4573260227485</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.3">
@@ -2723,7 +2841,7 @@
         <v>3.1028601038812176</v>
       </c>
       <c r="G5" s="4">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="H5" s="4">
         <v>736.50270198870771</v>
@@ -2736,19 +2854,19 @@
         <v>43</v>
       </c>
       <c r="L5" s="7">
-        <v>0.70248152838918376</v>
+        <v>7.0174170080653857</v>
       </c>
       <c r="N5" s="9" t="s">
         <v>67</v>
       </c>
       <c r="O5" s="10">
-        <v>1199.1350689643341</v>
+        <v>11978.456764170598</v>
       </c>
       <c r="Q5" s="13" t="s">
         <v>99</v>
       </c>
       <c r="R5" s="6">
-        <v>830.65281683265493</v>
+        <v>2963.220148019665</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.3">
@@ -2756,44 +2874,44 @@
         <v>4</v>
       </c>
       <c r="C6" s="4">
-        <v>976.11427576830124</v>
+        <v>976.21764828798996</v>
       </c>
       <c r="D6" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E6" s="4">
-        <v>1231.5688124201411</v>
+        <v>1231.6977516748684</v>
       </c>
       <c r="F6" s="7">
-        <v>3.1121411727413726</v>
+        <v>3.112273260172465</v>
       </c>
       <c r="G6" s="4">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="H6" s="4">
-        <v>613.82204441161923</v>
+        <v>613.91160179876624</v>
       </c>
       <c r="I6" s="4">
         <f t="shared" si="0"/>
-        <v>702.96427576830126</v>
+        <v>703.06764828798998</v>
       </c>
       <c r="K6" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L6" s="7">
-        <v>2.5004574163901339</v>
+        <v>24.984786638342218</v>
       </c>
       <c r="N6" s="9" t="s">
         <v>68</v>
       </c>
       <c r="O6" s="10">
-        <v>71.774211786387255</v>
+        <v>717.79640670783738</v>
       </c>
       <c r="Q6" s="13" t="s">
         <v>100</v>
       </c>
       <c r="R6" s="6">
-        <v>6850.0253590880538</v>
+        <v>48628.817203007362</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.3">
@@ -2801,44 +2919,44 @@
         <v>5</v>
       </c>
       <c r="C7" s="4">
-        <v>580.59332858273865</v>
+        <v>580.60739984606084</v>
       </c>
       <c r="D7" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E7" s="4">
-        <v>758.75704305028523</v>
+        <v>758.77316593152807</v>
       </c>
       <c r="F7" s="7">
-        <v>2.4934653765384365</v>
+        <v>2.493493145865219</v>
       </c>
       <c r="G7" s="4">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="H7" s="4">
-        <v>325.46846367966873</v>
+        <v>325.47630713613137</v>
       </c>
       <c r="I7" s="4">
         <f t="shared" si="0"/>
-        <v>307.44332858273867</v>
+        <v>307.45739984606087</v>
       </c>
       <c r="K7" s="9" t="s">
         <v>44</v>
       </c>
       <c r="L7" s="7">
-        <v>4.8493514799902702</v>
+        <v>48.505085709943238</v>
       </c>
       <c r="N7" s="9" t="s">
         <v>69</v>
       </c>
       <c r="O7" s="10">
-        <v>-386.40079286911646</v>
+        <v>-3864.0801901504483</v>
       </c>
       <c r="Q7" s="13" t="s">
         <v>105</v>
       </c>
       <c r="R7" s="6">
-        <v>2723.6906468307247</v>
+        <v>14404.513844749421</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.3">
@@ -2846,44 +2964,44 @@
         <v>6</v>
       </c>
       <c r="C8" s="4">
-        <v>435.43287838933054</v>
+        <v>435.4382571755965</v>
       </c>
       <c r="D8" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E8" s="4">
-        <v>591.19593244306282</v>
+        <v>591.20237940579909</v>
       </c>
       <c r="F8" s="7">
-        <v>2.1610419768753544</v>
+        <v>2.1610567826542426</v>
       </c>
       <c r="G8" s="4">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="H8" s="4">
-        <v>257.0193896819942</v>
+        <v>257.02142230175508</v>
       </c>
       <c r="I8" s="4">
         <f t="shared" si="0"/>
-        <v>162.28287838933056</v>
+        <v>162.28825717559653</v>
       </c>
       <c r="K8" s="9" t="s">
         <v>45</v>
       </c>
       <c r="L8" s="7">
-        <v>1.6756111060722243</v>
+        <v>16.757078652572897</v>
       </c>
       <c r="N8" s="9" t="s">
         <v>70</v>
       </c>
       <c r="O8" s="10">
-        <v>-188.73788675888972</v>
+        <v>-1887.2729900081154</v>
       </c>
       <c r="Q8" s="13" t="s">
         <v>104</v>
       </c>
       <c r="R8" s="6">
-        <v>150.85917384920415</v>
+        <v>125.94776703314032</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.3">
@@ -2891,44 +3009,44 @@
         <v>29</v>
       </c>
       <c r="C9" s="4">
-        <v>435.43287838933054</v>
+        <v>435.4382571755965</v>
       </c>
       <c r="D9" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E9" s="4">
-        <v>591.19593244306282</v>
+        <v>591.20237940579909</v>
       </c>
       <c r="F9" s="7">
-        <v>2.1610419768753544</v>
+        <v>2.1610567826542426</v>
       </c>
       <c r="G9" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H9" s="4">
-        <v>257.0193896819942</v>
+        <v>257.02142230175508</v>
       </c>
       <c r="I9" s="4">
         <f t="shared" si="0"/>
-        <v>162.28287838933056</v>
+        <v>162.28825717559653</v>
       </c>
       <c r="K9" s="9" t="s">
         <v>48</v>
       </c>
       <c r="L9" s="7">
-        <v>0.11033034486553291</v>
+        <v>1.1033708748874791</v>
       </c>
       <c r="N9" s="9" t="s">
         <v>71</v>
       </c>
       <c r="O9" s="10">
-        <v>-5.8779815586019524E-2</v>
+        <v>-0.58783407799472909</v>
       </c>
       <c r="Q9" s="13" t="s">
         <v>101</v>
       </c>
       <c r="R9" s="6">
-        <v>4757.3674529323171</v>
+        <v>54938.398428688655</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.3">
@@ -2936,44 +3054,44 @@
         <v>30</v>
       </c>
       <c r="C10" s="4">
-        <v>423.3557736165609</v>
+        <v>423.35913575479753</v>
       </c>
       <c r="D10" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E10" s="4">
-        <v>0.57659650223683723</v>
+        <v>0.57660060448894723</v>
       </c>
       <c r="F10" s="7">
-        <v>2.1270382629381421E-3</v>
+        <v>2.1270479527453361E-3</v>
       </c>
       <c r="G10" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H10" s="4">
-        <v>0.25257199616171355</v>
+        <v>0.25257320939780875</v>
       </c>
       <c r="I10" s="4">
         <f t="shared" si="0"/>
-        <v>150.20577361656092</v>
+        <v>150.20913575479756</v>
       </c>
       <c r="K10" s="9" t="s">
         <v>49</v>
       </c>
       <c r="L10" s="7">
-        <v>0.68666556854253946</v>
+        <v>6.8670753276560994</v>
       </c>
       <c r="N10" s="9" t="s">
         <v>72</v>
       </c>
       <c r="O10" s="10">
-        <v>1312.0360411963943</v>
+        <v>13100.101826786246</v>
       </c>
       <c r="Q10" s="13" t="s">
         <v>102</v>
       </c>
       <c r="R10" s="6">
-        <v>58326.910191272655</v>
+        <v>582641.93083540094</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.3">
@@ -2993,7 +3111,7 @@
         <v>1.8961819516546078E-3</v>
       </c>
       <c r="G11" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H11" s="4">
         <v>0.23185738014859708</v>
@@ -3006,19 +3124,19 @@
         <v>50</v>
       </c>
       <c r="L11" s="7">
-        <v>0.12544275752191905</v>
+        <v>1.2546499075118689</v>
       </c>
       <c r="N11" s="9" t="s">
         <v>73</v>
       </c>
       <c r="O11" s="10">
-        <v>71.715431970801234</v>
+        <v>717.20857262984271</v>
       </c>
       <c r="Q11" s="13" t="s">
         <v>103</v>
       </c>
       <c r="R11" s="6">
-        <v>101653.79754728591</v>
+        <v>1015444.9238863285</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.3">
@@ -3026,44 +3144,44 @@
         <v>32</v>
       </c>
       <c r="C12" s="4">
-        <v>346.62433578909861</v>
+        <v>346.62379557580101</v>
       </c>
       <c r="D12" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E12" s="4">
-        <v>0.46883148724964824</v>
+        <v>0.46883049635692192</v>
       </c>
       <c r="F12" s="7">
-        <v>1.844389053247172E-3</v>
+        <v>1.8443861945514714E-3</v>
       </c>
       <c r="G12" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H12" s="4">
-        <v>0.22907884304388729</v>
+        <v>0.22907870447128417</v>
       </c>
       <c r="I12" s="4">
         <f t="shared" si="0"/>
-        <v>73.474335789098632</v>
+        <v>73.473795575801034</v>
       </c>
       <c r="K12" s="9" t="s">
         <v>51</v>
       </c>
       <c r="L12" s="7">
-        <v>0.92243867092999143</v>
+        <v>9.2250961100554463</v>
       </c>
       <c r="N12" s="11" t="s">
         <v>74</v>
       </c>
       <c r="O12" s="12">
-        <v>1383.7514731671954</v>
+        <v>13817.310399416088</v>
       </c>
       <c r="Q12" s="13" t="s">
         <v>106</v>
       </c>
       <c r="R12" s="6">
-        <v>6084.4865460826932</v>
+        <v>60849.467667280827</v>
       </c>
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.3">
@@ -3071,38 +3189,38 @@
         <v>33</v>
       </c>
       <c r="C13" s="4">
-        <v>344.39458549639238</v>
+        <v>346.39737970663185</v>
       </c>
       <c r="D13" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E13" s="4">
-        <v>464.67130036926602</v>
+        <v>468.41449334690572</v>
       </c>
       <c r="F13" s="7">
-        <v>1.8323480555267959</v>
+        <v>1.8431856450668949</v>
       </c>
       <c r="G13" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H13" s="4">
-        <v>228.50867963383527</v>
+        <v>229.02064529009442</v>
       </c>
       <c r="I13" s="4">
         <f t="shared" si="0"/>
-        <v>71.244585496392403</v>
+        <v>73.247379706631875</v>
       </c>
       <c r="K13" s="9" t="s">
         <v>52</v>
       </c>
       <c r="L13" s="7">
-        <v>0.72305037797389082</v>
+        <v>7.2309456578341926</v>
       </c>
       <c r="Q13" s="13" t="s">
         <v>107</v>
       </c>
       <c r="R13" s="6">
-        <v>-14690.262623456645</v>
+        <v>-146905.37348517781</v>
       </c>
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.3">
@@ -3110,32 +3228,32 @@
         <v>34</v>
       </c>
       <c r="C14" s="4">
-        <v>435.43287838933054</v>
+        <v>435.4382571755965</v>
       </c>
       <c r="D14" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E14" s="4">
-        <v>591.19593244306282</v>
+        <v>591.20237940579909</v>
       </c>
       <c r="F14" s="7">
-        <v>2.1610419768753544</v>
+        <v>2.1610567826542426</v>
       </c>
       <c r="G14" s="4">
-        <v>2.0055144227139889</v>
+        <v>20.053649165005705</v>
       </c>
       <c r="H14" s="4">
-        <v>257.0193896819942</v>
+        <v>257.02142230175508</v>
       </c>
       <c r="I14" s="4">
         <f t="shared" si="0"/>
-        <v>162.28287838933056</v>
+        <v>162.28825717559653</v>
       </c>
       <c r="K14" s="9" t="s">
         <v>54</v>
       </c>
       <c r="L14" s="7">
-        <v>0.12767286098529926</v>
+        <v>1.2769418795914116</v>
       </c>
       <c r="N14" s="29" t="s">
         <v>75</v>
@@ -3145,7 +3263,7 @@
         <v>108</v>
       </c>
       <c r="R14" s="6">
-        <v>-7175.4747263768222</v>
+        <v>-71750.721988726538</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.3">
@@ -3165,7 +3283,7 @@
         <v>1.72122584179495</v>
       </c>
       <c r="G15" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H15" s="4">
         <v>224.33075530171814</v>
@@ -3178,19 +3296,19 @@
         <v>53</v>
       </c>
       <c r="L15" s="7">
-        <v>0.85072323895919011</v>
+        <v>8.5078875374256029</v>
       </c>
       <c r="N15" s="9" t="s">
         <v>80</v>
       </c>
       <c r="O15" s="10">
-        <v>7.7745474285568061</v>
+        <v>7.7745376749850683</v>
       </c>
       <c r="Q15" s="13" t="s">
         <v>109</v>
       </c>
       <c r="R15" s="6">
-        <v>-2.2347027849124075</v>
+        <v>-22.348393544019206</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.3">
@@ -3210,7 +3328,7 @@
         <v>1.7343043486568708</v>
       </c>
       <c r="G16" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H16" s="4">
         <v>268.76481394998945</v>
@@ -3223,19 +3341,19 @@
         <v>46</v>
       </c>
       <c r="L16" s="7">
-        <v>3.3258554014030113E-2</v>
+        <v>3.3257922587167379E-2</v>
       </c>
       <c r="N16" s="9" t="s">
         <v>81</v>
       </c>
       <c r="O16" s="10">
-        <v>52.471841055808</v>
+        <v>52.432314177470438</v>
       </c>
       <c r="Q16" s="13" t="s">
         <v>110</v>
       </c>
       <c r="R16" s="6">
-        <v>14936.432649657721</v>
+        <v>149375.6241707881</v>
       </c>
     </row>
     <row r="17" spans="2:25" x14ac:dyDescent="0.3">
@@ -3243,44 +3361,44 @@
         <v>9</v>
       </c>
       <c r="C17" s="4">
-        <v>547.68745921507718</v>
+        <v>547.69370647629023</v>
       </c>
       <c r="D17" s="5">
         <v>25</v>
       </c>
       <c r="E17" s="4">
-        <v>685.30539614040072</v>
+        <v>685.31357954095802</v>
       </c>
       <c r="F17" s="7">
-        <v>2.1800807088725671</v>
+        <v>2.180095650521598</v>
       </c>
       <c r="G17" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H17" s="4">
-        <v>345.45245543436323</v>
+        <v>345.4561839822619</v>
       </c>
       <c r="I17" s="4">
         <f t="shared" si="0"/>
-        <v>274.53745921507721</v>
+        <v>274.54370647629025</v>
       </c>
       <c r="K17" s="11" t="s">
         <v>55</v>
       </c>
       <c r="L17" s="16">
-        <v>-0.29815580239591893</v>
+        <v>-3.2808684015299132</v>
       </c>
       <c r="N17" s="9" t="s">
         <v>82</v>
       </c>
       <c r="O17" s="10">
-        <v>53.374586045417935</v>
+        <v>36.901993581878948</v>
       </c>
       <c r="Q17" s="13" t="s">
         <v>111</v>
       </c>
       <c r="R17" s="6">
-        <v>12158.725147647143</v>
+        <v>121456.51249638916</v>
       </c>
     </row>
     <row r="18" spans="2:25" x14ac:dyDescent="0.3">
@@ -3288,38 +3406,38 @@
         <v>10</v>
       </c>
       <c r="C18" s="4">
-        <v>547.68745921507718</v>
+        <v>547.69370647629023</v>
       </c>
       <c r="D18" s="5">
         <v>25</v>
       </c>
       <c r="E18" s="4">
-        <v>685.30539614040072</v>
+        <v>685.31357954095802</v>
       </c>
       <c r="F18" s="7">
-        <v>2.1800807088725671</v>
+        <v>2.180095650521598</v>
       </c>
       <c r="G18" s="4">
-        <v>2.0055144227139889</v>
+        <v>20.053649165005705</v>
       </c>
       <c r="H18" s="4">
-        <v>345.45245543436323</v>
+        <v>345.4561839822619</v>
       </c>
       <c r="I18" s="4">
         <f t="shared" si="0"/>
-        <v>274.53745921507721</v>
+        <v>274.54370647629025</v>
       </c>
       <c r="N18" s="9" t="s">
         <v>83</v>
       </c>
       <c r="O18" s="10">
-        <v>54.014275766007323</v>
+        <v>53.497400064021491</v>
       </c>
       <c r="Q18" s="13" t="s">
         <v>112</v>
       </c>
       <c r="R18" s="6">
-        <v>2143439.7108252258</v>
+        <v>21403100.470866345</v>
       </c>
     </row>
     <row r="19" spans="2:25" x14ac:dyDescent="0.3">
@@ -3327,26 +3445,26 @@
         <v>11</v>
       </c>
       <c r="C19" s="4">
-        <v>547.68745921507718</v>
+        <v>547.69370647629023</v>
       </c>
       <c r="D19" s="5">
         <v>25</v>
       </c>
       <c r="E19" s="4">
-        <v>685.30539614040072</v>
+        <v>685.31357954095802</v>
       </c>
       <c r="F19" s="7">
-        <v>2.1800807088725671</v>
+        <v>2.180095650521598</v>
       </c>
       <c r="G19" s="4">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="H19" s="4">
-        <v>345.45245543436323</v>
+        <v>345.4561839822619</v>
       </c>
       <c r="I19" s="4">
         <f t="shared" si="0"/>
-        <v>274.53745921507721</v>
+        <v>274.54370647629025</v>
       </c>
       <c r="K19" s="29" t="s">
         <v>58</v>
@@ -3356,13 +3474,13 @@
         <v>84</v>
       </c>
       <c r="O19" s="10">
-        <v>55.339933569630354</v>
+        <v>55.302895315550685</v>
       </c>
       <c r="Q19" s="13" t="s">
         <v>123</v>
       </c>
       <c r="R19" s="6">
-        <v>2503125.0768078174</v>
+        <v>24957461.093185224</v>
       </c>
     </row>
     <row r="20" spans="2:25" x14ac:dyDescent="0.3">
@@ -3370,38 +3488,38 @@
         <v>12</v>
       </c>
       <c r="C20" s="4">
-        <v>932.83907702081467</v>
+        <v>932.93660164805499</v>
       </c>
       <c r="D20" s="5">
         <v>25</v>
       </c>
       <c r="E20" s="4">
-        <v>1170.2405428635675</v>
+        <v>1170.3644353608943</v>
       </c>
       <c r="F20" s="7">
-        <v>2.8510501836319815</v>
+        <v>2.8511829889834948</v>
       </c>
       <c r="G20" s="4">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="H20" s="4">
-        <v>630.33805325801075</v>
+        <v>630.42234983978369</v>
       </c>
       <c r="I20" s="4">
         <f t="shared" si="0"/>
-        <v>659.68907702081469</v>
+        <v>659.78660164805501</v>
       </c>
       <c r="K20" s="13" t="s">
         <v>59</v>
       </c>
       <c r="L20" s="4">
-        <v>159.02185344711796</v>
+        <v>1128.9074473722574</v>
       </c>
       <c r="N20" s="9" t="s">
         <v>85</v>
       </c>
       <c r="O20" s="10">
-        <v>3.4933609588634824</v>
+        <v>3.4935322440475987</v>
       </c>
       <c r="Q20" s="28" t="s">
         <v>117</v>
@@ -3429,7 +3547,7 @@
         <v>-0.37994748587359245</v>
       </c>
       <c r="G21" s="4">
-        <v>1.7897056695309543</v>
+        <v>17.89815043892197</v>
       </c>
       <c r="H21" s="4">
         <v>0.52460446529691762</v>
@@ -3442,13 +3560,13 @@
         <v>60</v>
       </c>
       <c r="L21" s="4">
-        <v>63.229887799023224</v>
+        <v>334.39766563166074</v>
       </c>
       <c r="N21" s="9" t="s">
         <v>86</v>
       </c>
       <c r="O21" s="10">
-        <v>22.489305649899514</v>
+        <v>22.472364524327524</v>
       </c>
       <c r="Q21" s="22" t="s">
         <v>118</v>
@@ -3477,13 +3595,13 @@
         <v>-132.32179590986752</v>
       </c>
       <c r="F22" s="7">
-        <v>-0.37994748587359245</v>
+        <v>-0.37993175416231956</v>
       </c>
       <c r="G22" s="4">
-        <v>1.7897056695309543</v>
+        <v>17.89815043892197</v>
       </c>
       <c r="H22" s="4">
-        <v>0.55744775153482984</v>
+        <v>0.55275734181882941</v>
       </c>
       <c r="I22" s="4">
         <f t="shared" si="0"/>
@@ -3493,19 +3611,19 @@
         <v>61</v>
       </c>
       <c r="L22" s="4">
-        <v>21.287660768567079</v>
+        <v>71.721081948712694</v>
       </c>
       <c r="N22" s="9" t="s">
         <v>87</v>
       </c>
       <c r="O22" s="6">
-        <v>52.415130655682205</v>
+        <v>36.167181648495081</v>
       </c>
       <c r="Q22" s="23" t="s">
         <v>113</v>
       </c>
       <c r="R22" s="24">
-        <v>2505530.7763891984</v>
+        <v>24046.390970622553</v>
       </c>
       <c r="S22" s="23" t="s">
         <v>129</v>
@@ -3531,7 +3649,7 @@
         <v>-0.19317568283781225</v>
       </c>
       <c r="G23" s="4">
-        <v>1.7897056695309543</v>
+        <v>17.89815043892197</v>
       </c>
       <c r="H23" s="4">
         <v>6.518635522826691</v>
@@ -3544,19 +3662,19 @@
         <v>62</v>
       </c>
       <c r="L23" s="4">
-        <v>19.283425035580251</v>
+        <v>68.790513232882915</v>
       </c>
       <c r="N23" s="9" t="s">
         <v>88</v>
       </c>
       <c r="O23" s="6">
-        <v>23.133959295545651</v>
+        <v>22.917512377362197</v>
       </c>
       <c r="Q23" s="23" t="s">
         <v>114</v>
       </c>
       <c r="R23" s="24">
-        <v>4269212.9393934794</v>
+        <v>42594227.213088371</v>
       </c>
       <c r="S23" s="23" t="s">
         <v>128</v>
@@ -3582,7 +3700,7 @@
         <v>0.91173151933586583</v>
       </c>
       <c r="G24" s="4">
-        <v>1.7897056695309543</v>
+        <v>17.89815043892197</v>
       </c>
       <c r="H24" s="4">
         <v>60.765690527522125</v>
@@ -3595,25 +3713,25 @@
         <v>63</v>
       </c>
       <c r="L24" s="4">
-        <v>3.5021630107067545</v>
+        <v>2.9238501029143915</v>
       </c>
       <c r="N24" s="11" t="s">
         <v>89</v>
       </c>
       <c r="O24" s="15">
-        <v>23.136921933126388</v>
+        <v>22.919558145685983</v>
       </c>
       <c r="Q24" s="23" t="s">
         <v>115</v>
       </c>
       <c r="R24" s="24">
-        <v>202782.7454297191</v>
+        <v>2023167.7075799552</v>
       </c>
       <c r="S24" s="23" t="s">
         <v>127</v>
       </c>
       <c r="T24" s="27">
-        <v>2503125.0768078174</v>
+        <v>24957461.093185224</v>
       </c>
       <c r="V24" s="9"/>
       <c r="W24" s="9"/>
@@ -3625,37 +3743,39 @@
         <v>15</v>
       </c>
       <c r="C25" s="4">
-        <v>396.43287838933054</v>
+        <v>396.4382571755965</v>
       </c>
       <c r="D25" s="5">
         <v>31.569242975234697</v>
       </c>
       <c r="E25" s="4">
-        <v>383.09182021380718</v>
+        <v>383.09995906623425</v>
       </c>
       <c r="F25" s="7">
-        <v>1.1002468147744369</v>
+        <v>1.100267344850671</v>
       </c>
       <c r="G25" s="4">
-        <v>1.7897056695309543</v>
+        <v>17.89815043892197</v>
       </c>
       <c r="H25" s="4">
-        <v>74.651133136999675</v>
+        <v>74.65315094719746</v>
       </c>
       <c r="I25" s="4">
         <f t="shared" si="0"/>
-        <v>123.28287838933056</v>
+        <v>123.28825717559653</v>
       </c>
       <c r="K25" s="13" t="s">
         <v>64</v>
       </c>
       <c r="L25" s="4">
-        <v>110.44125389851233</v>
+        <v>1275.3830074447171</v>
       </c>
       <c r="Q25" s="9"/>
       <c r="R25" s="9"/>
       <c r="S25" s="9"/>
-      <c r="T25" s="26"/>
+      <c r="T25" s="26">
+        <v>48195801.93395783</v>
+      </c>
       <c r="V25" s="9"/>
       <c r="W25" s="9"/>
       <c r="X25" s="9"/>
@@ -3666,26 +3786,26 @@
         <v>16</v>
       </c>
       <c r="C26" s="4">
-        <v>368.13790080168786</v>
+        <v>368.14329244204333</v>
       </c>
       <c r="D26" s="5">
         <v>7.8923107438086744</v>
       </c>
       <c r="E26" s="4">
-        <v>342.98790088879446</v>
+        <v>342.99545725431005</v>
       </c>
       <c r="F26" s="7">
-        <v>1.119604713516257</v>
+        <v>1.1196252392794583</v>
       </c>
       <c r="G26" s="4">
-        <v>1.7897056695309543</v>
+        <v>17.89815043892197</v>
       </c>
       <c r="H26" s="4">
-        <v>28.775656302113202</v>
+        <v>28.777092911330342</v>
       </c>
       <c r="I26" s="4">
         <f t="shared" si="0"/>
-        <v>94.987900801687886</v>
+        <v>94.993292442043355</v>
       </c>
       <c r="N26" s="29" t="s">
         <v>76</v>
@@ -3717,7 +3837,7 @@
         <v>0.91018564327057938</v>
       </c>
       <c r="G27" s="4">
-        <v>1.7897056695309543</v>
+        <v>17.89815043892197</v>
       </c>
       <c r="H27" s="4">
         <v>19.876601402460075</v>
@@ -3759,7 +3879,7 @@
         <v>0.36719964130372146</v>
       </c>
       <c r="G28" s="4">
-        <v>34.591753259051274</v>
+        <v>345.9386726638856</v>
       </c>
       <c r="H28" s="4">
         <v>2.5073905791015251E-5</v>
@@ -3801,7 +3921,7 @@
         <v>0.43672528196163279</v>
       </c>
       <c r="G29" s="4">
-        <v>34.591753259051274</v>
+        <v>345.9386726638856</v>
       </c>
       <c r="H29" s="4">
         <v>0.17334706272843686</v>
@@ -3831,26 +3951,26 @@
         <v>39</v>
       </c>
       <c r="C30" s="4">
-        <v>304.03303316959324</v>
+        <v>304.03312670606874</v>
       </c>
       <c r="D30" s="5">
         <v>101.325</v>
       </c>
       <c r="E30" s="4">
-        <v>129.51335809758132</v>
+        <v>129.51374904828285</v>
       </c>
       <c r="F30" s="7">
-        <v>0.44888256955875044</v>
+        <v>0.44888385544072534</v>
       </c>
       <c r="G30" s="4">
-        <v>34.591753259051274</v>
+        <v>345.9386726638856</v>
       </c>
       <c r="H30" s="4">
-        <v>0.23949854144378332</v>
+        <v>0.23950610643450637</v>
       </c>
       <c r="I30" s="4">
         <f t="shared" si="0"/>
-        <v>30.883033169593261</v>
+        <v>30.883126706068765</v>
       </c>
       <c r="Q30" s="9"/>
       <c r="R30" s="9"/>
@@ -3867,26 +3987,26 @@
         <v>29</v>
       </c>
       <c r="C31" s="4">
-        <v>435.43287838933054</v>
+        <v>435.4382571755965</v>
       </c>
       <c r="D31" s="5">
         <v>9124.0875912408756</v>
       </c>
       <c r="E31" s="4">
-        <v>591.19593244282169</v>
+        <v>591.20237940555796</v>
       </c>
       <c r="F31" s="7">
-        <v>2.1610419768753544</v>
+        <v>2.1610567826542426</v>
       </c>
       <c r="G31" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H31" s="4">
-        <v>257.03321905731815</v>
+        <v>257.03525167707909</v>
       </c>
       <c r="I31" s="4">
         <f t="shared" si="0"/>
-        <v>162.28287838933056</v>
+        <v>162.28825717559653</v>
       </c>
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
@@ -3903,26 +4023,26 @@
         <v>30</v>
       </c>
       <c r="C32" s="4">
-        <v>423.3557736165609</v>
+        <v>423.35913575479753</v>
       </c>
       <c r="D32" s="5">
         <v>9124.0875912408756</v>
       </c>
       <c r="E32" s="4">
-        <v>576.59650223683718</v>
+        <v>576.60060448894728</v>
       </c>
       <c r="F32" s="7">
-        <v>2.1270382629381421</v>
+        <v>2.1270479527453361</v>
       </c>
       <c r="G32" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H32" s="4">
-        <v>252.57199616171354</v>
+        <v>252.57320939780874</v>
       </c>
       <c r="I32" s="4">
         <f t="shared" si="0"/>
-        <v>150.20577361656092</v>
+        <v>150.20913575479756</v>
       </c>
       <c r="Q32" s="9"/>
       <c r="R32" s="9"/>
@@ -3951,7 +4071,7 @@
         <v>1.8961819516546079</v>
       </c>
       <c r="G33" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H33" s="4">
         <v>231.85738014859709</v>
@@ -3975,26 +4095,26 @@
         <v>32</v>
       </c>
       <c r="C34" s="4">
-        <v>346.62433578909861</v>
+        <v>346.62379557580101</v>
       </c>
       <c r="D34" s="5">
         <v>9124.0875912408756</v>
       </c>
       <c r="E34" s="4">
-        <v>468.83148724964826</v>
+        <v>468.83049635692191</v>
       </c>
       <c r="F34" s="7">
-        <v>1.8443890532471721</v>
+        <v>1.8443861945514715</v>
       </c>
       <c r="G34" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H34" s="4">
-        <v>229.07884304388728</v>
+        <v>229.07870447128417</v>
       </c>
       <c r="I34" s="4">
         <f t="shared" si="0"/>
-        <v>73.474335789098632</v>
+        <v>73.473795575801034</v>
       </c>
     </row>
     <row r="35" spans="2:25" x14ac:dyDescent="0.3">
@@ -4035,16 +4155,16 @@
         <v>0.101325</v>
       </c>
       <c r="E36" s="4">
-        <v>453.10722153513228</v>
+        <v>453.10667720162991</v>
       </c>
       <c r="F36" s="7">
-        <v>3.9723323134988857</v>
+        <v>3.9723306469545014</v>
       </c>
       <c r="G36" s="4">
         <v>1.1599999999999999</v>
       </c>
       <c r="H36" s="4">
-        <v>1.3091135519945019</v>
+        <v>1.3090660987003904</v>
       </c>
       <c r="I36" s="4">
         <f t="shared" si="0"/>
@@ -4056,26 +4176,26 @@
         <v>32</v>
       </c>
       <c r="C37" s="4">
-        <v>346.62433578909861</v>
+        <v>346.62379557580101</v>
       </c>
       <c r="D37" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E37" s="4">
-        <v>468.83148724964826</v>
+        <v>468.83049635692191</v>
       </c>
       <c r="F37" s="7">
-        <v>1.8443890532471721</v>
+        <v>1.8443861945514715</v>
       </c>
       <c r="G37" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H37" s="4">
-        <v>229.07884304388728</v>
+        <v>229.07870447128417</v>
       </c>
       <c r="I37" s="4">
         <f t="shared" si="0"/>
-        <v>73.474335789098632</v>
+        <v>73.473795575801034</v>
       </c>
     </row>
     <row r="38" spans="2:25" x14ac:dyDescent="0.3">
@@ -4083,26 +4203,26 @@
         <v>33</v>
       </c>
       <c r="C38" s="4">
-        <v>344.39458549639238</v>
+        <v>346.39737970663185</v>
       </c>
       <c r="D38" s="5">
         <v>9.1240875912408761</v>
       </c>
       <c r="E38" s="4">
-        <v>464.67130036926602</v>
+        <v>468.41449334690572</v>
       </c>
       <c r="F38" s="7">
-        <v>1.8323480555267959</v>
+        <v>1.8431856450668949</v>
       </c>
       <c r="G38" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H38" s="4">
-        <v>228.50867963383527</v>
+        <v>229.02064529009442</v>
       </c>
       <c r="I38" s="4">
         <f t="shared" si="0"/>
-        <v>71.244585496392403</v>
+        <v>73.247379706631875</v>
       </c>
     </row>
     <row r="39" spans="2:25" x14ac:dyDescent="0.3">
@@ -4110,26 +4230,26 @@
         <v>33</v>
       </c>
       <c r="C39" s="4">
-        <v>344.39458549639238</v>
+        <v>346.39737970663185</v>
       </c>
       <c r="D39" s="5">
         <v>9124.0875912408756</v>
       </c>
       <c r="E39" s="4">
-        <v>464.67130036356895</v>
+        <v>468.41449334022548</v>
       </c>
       <c r="F39" s="7">
-        <v>1.8323480555267959</v>
+        <v>1.8431856450668949</v>
       </c>
       <c r="G39" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H39" s="4">
-        <v>228.5086796281382</v>
+        <v>229.02064528341415</v>
       </c>
       <c r="I39" s="4">
         <f t="shared" si="0"/>
-        <v>71.244585496392403</v>
+        <v>73.247379706631875</v>
       </c>
     </row>
     <row r="40" spans="2:25" x14ac:dyDescent="0.3">
@@ -4149,7 +4269,7 @@
         <v>1.72122584179495</v>
       </c>
       <c r="G40" s="4">
-        <v>7.9944855772860111</v>
+        <v>79.946350834994291</v>
       </c>
       <c r="H40" s="4">
         <v>224.34458467728319</v>
@@ -4176,7 +4296,7 @@
         <v>0.36719964130372146</v>
       </c>
       <c r="G41" s="4">
-        <v>2.8698525619149113E-3</v>
+        <v>1.9801295635402501E-2</v>
       </c>
       <c r="H41" s="4">
         <v>2.5073905791015251E-5</v>
@@ -4191,26 +4311,26 @@
         <v>20</v>
       </c>
       <c r="C42" s="4">
-        <v>343.39458549639238</v>
+        <v>345.39737970663185</v>
       </c>
       <c r="D42" s="5">
         <v>101.325</v>
       </c>
       <c r="E42" s="4">
-        <v>294.14738747128831</v>
+        <v>302.54072536549046</v>
       </c>
       <c r="F42" s="7">
-        <v>0.95807613660276081</v>
+        <v>0.98244738595667158</v>
       </c>
       <c r="G42" s="4">
-        <v>2.8698525619149113E-3</v>
+        <v>1.9801295635402501E-2</v>
       </c>
       <c r="H42" s="4">
-        <v>13.057465900979093</v>
+        <v>14.184515800312743</v>
       </c>
       <c r="I42" s="4">
         <f t="shared" si="0"/>
-        <v>70.244585496392403</v>
+        <v>72.247379706631875</v>
       </c>
     </row>
   </sheetData>
@@ -4231,6 +4351,540 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9BBA90F-813A-493D-869A-57A3178EDC43}">
+  <dimension ref="A1:M26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2">
+        <v>5.1731913323680587E-2</v>
+      </c>
+      <c r="C2">
+        <v>3914.1005686252538</v>
+      </c>
+      <c r="E2" t="s">
+        <v>66</v>
+      </c>
+      <c r="F2">
+        <v>2503.1935161652605</v>
+      </c>
+      <c r="G2">
+        <v>154.12694860114715</v>
+      </c>
+      <c r="H2">
+        <v>7.9732819458779174</v>
+      </c>
+      <c r="I2">
+        <v>99.682486963754258</v>
+      </c>
+      <c r="K2" s="31">
+        <v>0.34909743323706877</v>
+      </c>
+      <c r="L2" s="31">
+        <v>0.91088630043789787</v>
+      </c>
+      <c r="M2" s="31">
+        <v>0.27584737694031641</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B3">
+        <v>5.1731913323680594E-2</v>
+      </c>
+      <c r="C3">
+        <v>3550.5739373103711</v>
+      </c>
+      <c r="E3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3">
+        <v>888.25965020835133</v>
+      </c>
+      <c r="G3">
+        <v>280.65325482354871</v>
+      </c>
+      <c r="H3">
+        <v>13.912184589022015</v>
+      </c>
+      <c r="I3">
+        <v>98.457922975156208</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B4">
+        <v>4.9570722412497346E-2</v>
+      </c>
+      <c r="C4">
+        <v>3650.8970996336493</v>
+      </c>
+      <c r="E4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F4">
+        <v>27.111169102991425</v>
+      </c>
+      <c r="G4">
+        <v>311.73934843303778</v>
+      </c>
+      <c r="H4">
+        <v>85.992481554336806</v>
+      </c>
+      <c r="I4">
+        <v>23.970198084171948</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B5">
+        <v>4.9570722412497353E-2</v>
+      </c>
+      <c r="C5">
+        <v>3043.2041598578253</v>
+      </c>
+      <c r="E5" t="s">
+        <v>70</v>
+      </c>
+      <c r="F5">
+        <v>6.8005339576619255</v>
+      </c>
+      <c r="G5">
+        <v>113.83330527634081</v>
+      </c>
+      <c r="H5">
+        <v>31.400618668924892</v>
+      </c>
+      <c r="I5">
+        <v>17.801907770000021</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>207</v>
+      </c>
+      <c r="B6">
+        <v>4.9570722412497326E-2</v>
+      </c>
+      <c r="C6">
+        <v>1613.4095672889889</v>
+      </c>
+      <c r="E6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6">
+        <v>10.532285533619728</v>
+      </c>
+      <c r="G6">
+        <v>346.91288051130834</v>
+      </c>
+      <c r="H6">
+        <v>17.19672210114593</v>
+      </c>
+      <c r="I6">
+        <v>37.98291548095186</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>208</v>
+      </c>
+      <c r="B7">
+        <v>4.9570722412497346E-2</v>
+      </c>
+      <c r="C7">
+        <v>1274.0737578985556</v>
+      </c>
+      <c r="E7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7">
+        <v>5.1377091499340155</v>
+      </c>
+      <c r="G7">
+        <v>714.29330882120883</v>
+      </c>
+      <c r="H7">
+        <v>35.40803533268037</v>
+      </c>
+      <c r="I7">
+        <v>12.67138935415778</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B8">
+        <v>5.6564567203107923E-5</v>
+      </c>
+      <c r="C8">
+        <v>1.01445300323212</v>
+      </c>
+      <c r="E8" t="s">
+        <v>229</v>
+      </c>
+      <c r="F8">
+        <v>2.0715042857927268</v>
+      </c>
+      <c r="G8">
+        <v>908.7639387171597</v>
+      </c>
+      <c r="H8">
+        <v>45.048084944636095</v>
+      </c>
+      <c r="I8">
+        <v>4.3962698309241492</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B9">
+        <v>5.09160848747457E-2</v>
+      </c>
+      <c r="C9">
+        <v>1094.0220068462638</v>
+      </c>
+      <c r="E9" t="s">
+        <v>230</v>
+      </c>
+      <c r="F9">
+        <v>14.87368048383521</v>
+      </c>
+      <c r="G9">
+        <v>103.30018156282743</v>
+      </c>
+      <c r="H9">
+        <v>128.39674035958012</v>
+      </c>
+      <c r="I9">
+        <v>10.381543096108523</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>211</v>
+      </c>
+      <c r="B10">
+        <v>5.2085507350043407E-2</v>
+      </c>
+      <c r="C10">
+        <v>1438.4955253866315</v>
+      </c>
+      <c r="E10" t="s">
+        <v>231</v>
+      </c>
+      <c r="F10">
+        <v>3.0925794872948675E-2</v>
+      </c>
+      <c r="G10">
+        <v>8.3949658717157039E-2</v>
+      </c>
+      <c r="H10">
+        <v>2.3157293152162538E-2</v>
+      </c>
+      <c r="I10">
+        <v>57.182006431640112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>212</v>
+      </c>
+      <c r="B11">
+        <v>0.11301051802733234</v>
+      </c>
+      <c r="C11">
+        <v>782.89811933408907</v>
+      </c>
+      <c r="E11" t="s">
+        <v>232</v>
+      </c>
+      <c r="F11">
+        <v>0.64803276948092892</v>
+      </c>
+      <c r="G11">
+        <v>422.82153795985045</v>
+      </c>
+      <c r="H11">
+        <v>525.54512883262078</v>
+      </c>
+      <c r="I11">
+        <v>0.12315492043033435</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>213</v>
+      </c>
+      <c r="B12">
+        <v>6.4303195245009187E-2</v>
+      </c>
+      <c r="C12">
+        <v>2221.3936447207207</v>
+      </c>
+      <c r="E12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F12">
+        <v>0.12782276758325392</v>
+      </c>
+      <c r="G12">
+        <v>3.1475926729674328</v>
+      </c>
+      <c r="H12">
+        <v>0.15602844265927923</v>
+      </c>
+      <c r="I12">
+        <v>45.031609156796392</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>214</v>
+      </c>
+      <c r="B13">
+        <v>5.8083608929057957E-2</v>
+      </c>
+      <c r="C13">
+        <v>3661.7205228231765</v>
+      </c>
+      <c r="E13" t="s">
+        <v>233</v>
+      </c>
+      <c r="F13">
+        <v>2.9067425972745697</v>
+      </c>
+      <c r="G13">
+        <v>373.5531104491323</v>
+      </c>
+      <c r="H13">
+        <v>2.1129870019932807E-2</v>
+      </c>
+      <c r="I13">
+        <v>99.278320000069613</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>215</v>
+      </c>
+      <c r="B14">
+        <v>4.9570722412497333E-2</v>
+      </c>
+      <c r="C14">
+        <v>255.49828151238043</v>
+      </c>
+      <c r="E14" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="F14" s="30">
+        <v>38.53098439483005</v>
+      </c>
+      <c r="G14" s="30">
+        <v>456.8011680060402</v>
+      </c>
+      <c r="H14" s="30">
+        <v>126.00740397773897</v>
+      </c>
+      <c r="I14" s="30">
+        <v>23.417625987428071</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>216</v>
+      </c>
+      <c r="B15">
+        <v>4.9570722412497367E-2</v>
+      </c>
+      <c r="C15">
+        <v>1018.5754763861755</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>217</v>
+      </c>
+      <c r="B16">
+        <v>4.9570722412497367E-2</v>
+      </c>
+      <c r="C16">
+        <v>0.90783853130662884</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>218</v>
+      </c>
+      <c r="B17">
+        <v>5.6564567203115594E-5</v>
+      </c>
+      <c r="C17">
+        <v>1.0356612988898828</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>228</v>
+      </c>
+      <c r="B18">
+        <v>2E-3</v>
+      </c>
+      <c r="C18">
+        <v>9.9299164260424743E-10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>219</v>
+      </c>
+      <c r="B19">
+        <v>10.424510362939218</v>
+      </c>
+      <c r="C19">
+        <v>2.9279508939251864</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>220</v>
+      </c>
+      <c r="B20">
+        <v>1.2429478672454113</v>
+      </c>
+      <c r="C20">
+        <v>1660.7689273524077</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>221</v>
+      </c>
+      <c r="B21">
+        <v>1.2429478672454113</v>
+      </c>
+      <c r="C21">
+        <v>640.18867415890122</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>222</v>
+      </c>
+      <c r="B22">
+        <v>68.250720909430768</v>
+      </c>
+      <c r="C22">
+        <v>640.83670692838211</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>223</v>
+      </c>
+      <c r="B23">
+        <v>64.794110996165372</v>
+      </c>
+      <c r="C23">
+        <v>641.029785211746</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>224</v>
+      </c>
+      <c r="B24">
+        <v>0.91088630043789787</v>
+      </c>
+      <c r="C24">
+        <v>236.37108787388058</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>225</v>
+      </c>
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="B26" s="30">
+        <v>0.27584737694031641</v>
+      </c>
+      <c r="C26" s="30">
+        <v>197.84010347905053</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63E0693F-D387-4367-8A44-8725A6CA7BA7}">
   <dimension ref="A1:AF33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
environ Mensaje de commit
</commit_message>
<xml_diff>
--- a/Salidas.xlsx
+++ b/Salidas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acih0\Documents\CODIGO\tes2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A858FA-2336-44E5-A497-0C75CCEB9BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86FCA34-9C00-4775-A2B5-3CE814481FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3336" yWindow="3540" windowWidth="17280" windowHeight="9420" xr2:uid="{C4CE93A3-0861-4D2C-B953-37868A8DFB1C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{C4CE93A3-0861-4D2C-B953-37868A8DFB1C}"/>
   </bookViews>
   <sheets>
     <sheet name="T" sheetId="3" r:id="rId1"/>
@@ -2531,10 +2531,10 @@
         <v>0.27721683884119408</v>
       </c>
       <c r="F29" s="16">
-        <v>1.3066538362716359E-2</v>
+        <v>1.2725895991014955E-2</v>
       </c>
       <c r="G29" s="16">
-        <v>0.76196895766048367</v>
+        <v>0.74329834926752969</v>
       </c>
       <c r="H29" s="16">
         <v>21.757787473165259</v>
@@ -2566,10 +2566,10 @@
         <v>0.29141583095469492</v>
       </c>
       <c r="F30" s="16">
-        <v>1.2891638164129249E-2</v>
+        <v>1.256705583287248E-2</v>
       </c>
       <c r="G30" s="16">
-        <v>0.75238267777592416</v>
+        <v>0.73459232019974063</v>
       </c>
       <c r="H30" s="16">
         <v>22.620890157848095</v>
@@ -2601,10 +2601,10 @@
         <v>0.30082239580281539</v>
       </c>
       <c r="F31" s="16">
-        <v>1.278733576486221E-2</v>
+        <v>1.2460487945338345E-2</v>
       </c>
       <c r="G31" s="16">
-        <v>0.74666586327209783</v>
+        <v>0.72875133428399475</v>
       </c>
       <c r="H31" s="16">
         <v>23.183143546879993</v>
@@ -2636,10 +2636,10 @@
         <v>0.30563943460760568</v>
       </c>
       <c r="F32" s="16">
-        <v>1.2743286995087122E-2</v>
+        <v>1.2396637952335364E-2</v>
       </c>
       <c r="G32" s="16">
-        <v>0.7442515502007252</v>
+        <v>0.72525171616750128</v>
       </c>
       <c r="H32" s="16">
         <v>23.469051190883171</v>
@@ -2671,10 +2671,10 @@
         <v>0.30600947271635609</v>
       </c>
       <c r="F33" s="16">
-        <v>1.2760809080769826E-2</v>
+        <v>1.2373819823211687E-2</v>
       </c>
       <c r="G33" s="16">
-        <v>0.74521193571699418</v>
+        <v>0.72400105451023267</v>
       </c>
       <c r="H33" s="16">
         <v>23.49293753748929</v>
@@ -2706,10 +2706,10 @@
         <v>0.30204684930766268</v>
       </c>
       <c r="F34" s="16">
-        <v>1.2855676451430006E-2</v>
+        <v>1.2399204794170266E-2</v>
       </c>
       <c r="G34" s="16">
-        <v>0.75041161630287867</v>
+        <v>0.72539240476847233</v>
       </c>
       <c r="H34" s="16">
         <v>23.261899200976021</v>
@@ -2741,10 +2741,10 @@
         <v>0.29386112662101954</v>
       </c>
       <c r="F35" s="16">
-        <v>1.3075242228025856E-2</v>
+        <v>1.2498061236008415E-2</v>
       </c>
       <c r="G35" s="16">
-        <v>0.76244601651809718</v>
+        <v>0.73081072634562128</v>
       </c>
       <c r="H35" s="16">
         <v>22.777686776908567</v>
@@ -2776,10 +2776,10 @@
         <v>0.28157430810541256</v>
       </c>
       <c r="F36" s="16">
-        <v>1.3578355310744016E-2</v>
+        <v>1.2758135640936705E-2</v>
       </c>
       <c r="G36" s="16">
-        <v>0.79002164458187951</v>
+        <v>0.74506540447974079</v>
       </c>
       <c r="H36" s="16">
         <v>22.037942778693676</v>
@@ -2811,10 +2811,10 @@
         <v>0.26533370011538154</v>
       </c>
       <c r="F37" s="16">
-        <v>1.5671120364137446E-2</v>
+        <v>1.390700110545017E-2</v>
       </c>
       <c r="G37" s="16">
-        <v>0.90472609715837349</v>
+        <v>0.80803472058972381</v>
       </c>
       <c r="H37" s="16">
         <v>21.037063645279886</v>
@@ -2846,10 +2846,10 @@
         <v>0.29386112662101954</v>
       </c>
       <c r="F38" s="18">
-        <v>1.3075242228025856E-2</v>
+        <v>1.2498061236008415E-2</v>
       </c>
       <c r="G38" s="18">
-        <v>0.76244601651809718</v>
+        <v>0.73081072634562128</v>
       </c>
       <c r="H38" s="18">
         <v>22.777686776908567</v>
@@ -3619,10 +3619,10 @@
         <v>0.26242431235563907</v>
       </c>
       <c r="F29" s="16">
-        <v>1.2687298913338699E-2</v>
+        <v>1.2211101410757789E-2</v>
       </c>
       <c r="G29" s="16">
-        <v>0.74118284344009411</v>
+        <v>0.71508245832363448</v>
       </c>
       <c r="H29" s="16">
         <v>20.8250053094837</v>
@@ -3654,10 +3654,10 @@
         <v>0.26498555144485081</v>
       </c>
       <c r="F30" s="16">
-        <v>1.3781762480049234E-2</v>
+        <v>1.2848659426448708E-2</v>
       </c>
       <c r="G30" s="16">
-        <v>0.8011703915314986</v>
+        <v>0.75002701316365372</v>
       </c>
       <c r="H30" s="16">
         <v>21.010323870069069</v>
@@ -3689,10 +3689,10 @@
         <v>0.26634915185839914</v>
       </c>
       <c r="F31" s="16">
-        <v>1.3238832473157039E-2</v>
+        <v>1.2569616257764678E-2</v>
       </c>
       <c r="G31" s="16">
-        <v>0.77141239785373727</v>
+        <v>0.734732657088082</v>
       </c>
       <c r="H31" s="16">
         <v>21.120968205447276</v>
@@ -3724,10 +3724,10 @@
         <v>0.26699299315765596</v>
       </c>
       <c r="F32" s="16">
-        <v>1.2331820908740496E-2</v>
+        <v>1.2084861351781972E-2</v>
       </c>
       <c r="G32" s="16">
-        <v>0.72169909400806664</v>
+        <v>0.70816324069116998</v>
       </c>
       <c r="H32" s="16">
         <v>21.188960488161513</v>
@@ -3759,10 +3759,10 @@
         <v>0.26715706725652344</v>
       </c>
       <c r="F33" s="16">
-        <v>1.1959199986815333E-2</v>
+        <v>1.1896018768568203E-2</v>
       </c>
       <c r="G33" s="16">
-        <v>0.70127574127734837</v>
+        <v>0.69781277870522329</v>
       </c>
       <c r="H33" s="16">
         <v>21.228220514190312</v>
@@ -3794,10 +3794,10 @@
         <v>0.26698424761118889</v>
       </c>
       <c r="F34" s="16">
-        <v>1.175660043776486E-2</v>
+        <v>1.1800413306798704E-2</v>
       </c>
       <c r="G34" s="16">
-        <v>0.69017125999389195</v>
+        <v>0.69257264334563695</v>
       </c>
       <c r="H34" s="16">
         <v>21.246913286205405</v>
@@ -4665,10 +4665,10 @@
         <v>0.17164807793559991</v>
       </c>
       <c r="F29" s="16">
-        <v>2.0341675998230901E-2</v>
+        <v>1.6757024969993196E-2</v>
       </c>
       <c r="G29" s="16">
-        <v>1.1607192514630356</v>
+        <v>0.96424452860532706</v>
       </c>
       <c r="H29" s="16">
         <v>14.757340342055347</v>
@@ -4700,10 +4700,10 @@
         <v>0.1888468926271184</v>
       </c>
       <c r="F30" s="16">
-        <v>1.978432924799594E-2</v>
+        <v>1.6384759955406843E-2</v>
       </c>
       <c r="G30" s="16">
-        <v>1.1301710760826573</v>
+        <v>0.94384068315584913</v>
       </c>
       <c r="H30" s="16">
         <v>15.983919810375957</v>
@@ -4735,10 +4735,10 @@
         <v>0.20480986996949019</v>
       </c>
       <c r="F31" s="16">
-        <v>1.9555506784251827E-2</v>
+        <v>1.6208407990483766E-2</v>
       </c>
       <c r="G31" s="16">
-        <v>1.1176293168448426</v>
+        <v>0.93417483195841522</v>
       </c>
       <c r="H31" s="16">
         <v>17.091203390183175</v>
@@ -4770,10 +4770,10 @@
         <v>0.21966556495623429</v>
       </c>
       <c r="F32" s="16">
-        <v>1.9780145140133622E-2</v>
+        <v>1.6294029696723257E-2</v>
       </c>
       <c r="G32" s="16">
-        <v>1.1299417451307239</v>
+        <v>0.93886775767740172</v>
       </c>
       <c r="H32" s="16">
         <v>18.095784881552312</v>
@@ -4805,10 +4805,10 @@
         <v>0.23352530431347171</v>
       </c>
       <c r="F33" s="16">
-        <v>2.1278787193004869E-2</v>
+        <v>1.7096731860174904E-2</v>
       </c>
       <c r="G33" s="16">
-        <v>1.2120823160485967</v>
+        <v>0.98286386325618658</v>
       </c>
       <c r="H33" s="16">
         <v>19.011318909297625</v>
@@ -4840,10 +4840,10 @@
         <v>0.24648595905073192</v>
       </c>
       <c r="F34" s="16">
-        <v>1.9465300659532975E-2</v>
+        <v>1.6058055835609431E-2</v>
       </c>
       <c r="G34" s="16">
-        <v>1.1126851191490024</v>
+        <v>0.92593403034975297</v>
       </c>
       <c r="H34" s="16">
         <v>19.849141217844313</v>
@@ -4875,10 +4875,10 @@
         <v>0.25863227729297766</v>
       </c>
       <c r="F35" s="16">
-        <v>1.6483802014683472E-2</v>
+        <v>1.4372241813136767E-2</v>
       </c>
       <c r="G35" s="16">
-        <v>0.94926917842480119</v>
+        <v>0.83353456377802626</v>
       </c>
       <c r="H35" s="16">
         <v>20.618744692025714</v>
@@ -5746,10 +5746,10 @@
         <v>0.21752070053998984</v>
       </c>
       <c r="F29" s="16">
-        <v>1.3347972360860334E-2</v>
+        <v>1.2820307346803273E-2</v>
       </c>
       <c r="G29" s="16">
-        <v>0.77739435509875499</v>
+        <v>0.74847303567828738</v>
       </c>
       <c r="H29" s="16">
         <v>17.986004189136761</v>
@@ -5781,10 +5781,10 @@
         <v>0.22887252850425274</v>
       </c>
       <c r="F30" s="16">
-        <v>1.3291196355712501E-2</v>
+        <v>1.2732527471849048E-2</v>
       </c>
       <c r="G30" s="16">
-        <v>0.77428246225660224</v>
+        <v>0.74366182073204634</v>
       </c>
       <c r="H30" s="16">
         <v>18.729554829407846</v>
@@ -5816,10 +5816,10 @@
         <v>0.23858500738232519</v>
       </c>
       <c r="F31" s="16">
-        <v>1.3259884166837736E-2</v>
+        <v>1.2670697653095902E-2</v>
       </c>
       <c r="G31" s="16">
-        <v>0.77256624118437633</v>
+        <v>0.74027292836618641</v>
       </c>
       <c r="H31" s="16">
         <v>19.356136135287894</v>
@@ -5851,10 +5851,10 @@
         <v>0.24698231842324175</v>
       </c>
       <c r="F32" s="16">
-        <v>1.3246821447386169E-2</v>
+        <v>1.262745197607002E-2</v>
       </c>
       <c r="G32" s="16">
-        <v>0.77185027353123592</v>
+        <v>0.73790263280839785</v>
       </c>
       <c r="H32" s="16">
         <v>19.890850554306937</v>
@@ -5886,10 +5886,10 @@
         <v>0.25430934115195086</v>
       </c>
       <c r="F33" s="16">
-        <v>1.3247346740240681E-2</v>
+        <v>1.259800766538546E-2</v>
       </c>
       <c r="G33" s="16">
-        <v>0.77187906483259183</v>
+        <v>0.73628879013977711</v>
       </c>
       <c r="H33" s="16">
         <v>20.35216278034363</v>
@@ -5921,10 +5921,10 @@
         <v>0.26075436728817891</v>
       </c>
       <c r="F34" s="16">
-        <v>1.3258314031391686E-2</v>
+        <v>1.257912344780103E-2</v>
       </c>
       <c r="G34" s="16">
-        <v>0.77248018206057834</v>
+        <v>0.73525374617397443</v>
       </c>
       <c r="H34" s="16">
         <v>20.753941271896004</v>
@@ -5956,10 +5956,10 @@
         <v>0.26646417225585195</v>
       </c>
       <c r="F35" s="16">
-        <v>1.3277549695321836E-2</v>
+        <v>1.2568539303476595E-2</v>
       </c>
       <c r="G35" s="16">
-        <v>0.77353448880058984</v>
+        <v>0.73467362922355217</v>
       </c>
       <c r="H35" s="16">
         <v>21.106712178216604</v>
@@ -6124,7 +6124,7 @@
         <v>98</v>
       </c>
       <c r="R4" s="5">
-        <v>6393.9317076702955</v>
+        <v>3564.7236360481061</v>
       </c>
     </row>
     <row r="5" spans="2:18" x14ac:dyDescent="0.3">
@@ -6169,7 +6169,7 @@
         <v>99</v>
       </c>
       <c r="R5" s="5">
-        <v>7601.6529923868393</v>
+        <v>4238.0484080694978</v>
       </c>
     </row>
     <row r="6" spans="2:18" x14ac:dyDescent="0.3">
@@ -6214,7 +6214,7 @@
         <v>100</v>
       </c>
       <c r="R6" s="5">
-        <v>315741.08336552046</v>
+        <v>176030.92341356995</v>
       </c>
     </row>
     <row r="7" spans="2:18" x14ac:dyDescent="0.3">
@@ -6259,7 +6259,7 @@
         <v>105</v>
       </c>
       <c r="R7" s="5">
-        <v>82524.716891440621</v>
+        <v>46008.906930956873</v>
       </c>
     </row>
     <row r="8" spans="2:18" x14ac:dyDescent="0.3">
@@ -6304,7 +6304,7 @@
         <v>104</v>
       </c>
       <c r="R8" s="5">
-        <v>619.2519616594775</v>
+        <v>345.24330338852025</v>
       </c>
     </row>
     <row r="9" spans="2:18" x14ac:dyDescent="0.3">
@@ -6349,7 +6349,7 @@
         <v>101</v>
       </c>
       <c r="R9" s="5">
-        <v>47345560.666325219</v>
+        <v>26395940.226689368</v>
       </c>
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.3">
@@ -6394,7 +6394,7 @@
         <v>102</v>
       </c>
       <c r="R10" s="5">
-        <v>4474545.5721388133</v>
+        <v>7331176.3611313887</v>
       </c>
     </row>
     <row r="11" spans="2:18" x14ac:dyDescent="0.3">
@@ -6439,7 +6439,7 @@
         <v>103</v>
       </c>
       <c r="R11" s="5">
-        <v>7798365.2522427328</v>
+        <v>12776982.616668882</v>
       </c>
     </row>
     <row r="12" spans="2:18" x14ac:dyDescent="0.3">
@@ -6484,7 +6484,7 @@
         <v>106</v>
       </c>
       <c r="R12" s="5">
-        <v>493351.64968492277</v>
+        <v>808316.26219563605</v>
       </c>
     </row>
     <row r="13" spans="2:18" x14ac:dyDescent="0.3">
@@ -6523,7 +6523,7 @@
         <v>107</v>
       </c>
       <c r="R13" s="5">
-        <v>1128196.8455462928</v>
+        <v>1848458.1085221746</v>
       </c>
     </row>
     <row r="14" spans="2:18" x14ac:dyDescent="0.3">
@@ -6566,7 +6566,7 @@
         <v>108</v>
       </c>
       <c r="R14" s="5">
-        <v>551027.75543821603</v>
+        <v>902813.83659368719</v>
       </c>
     </row>
     <row r="15" spans="2:18" x14ac:dyDescent="0.3">
@@ -6611,7 +6611,7 @@
         <v>109</v>
       </c>
       <c r="R15" s="5">
-        <v>580.12586564866683</v>
+        <v>950.48870643001896</v>
       </c>
     </row>
     <row r="16" spans="2:18" x14ac:dyDescent="0.3">
@@ -6750,7 +6750,7 @@
       </c>
       <c r="V18" s="5">
         <f>R23-R9-R6</f>
-        <v>209111725.97569132</v>
+        <v>218858501.26033798</v>
       </c>
     </row>
     <row r="19" spans="2:25" x14ac:dyDescent="0.3">
@@ -6793,7 +6793,7 @@
         <v>122</v>
       </c>
       <c r="R19" s="5">
-        <v>287036742.70045835</v>
+        <v>275127059.32777882</v>
       </c>
     </row>
     <row r="20" spans="2:25" x14ac:dyDescent="0.3">
@@ -6838,7 +6838,7 @@
         <v>250</v>
       </c>
       <c r="R20">
-        <v>1.3892468513357714</v>
+        <v>0.77452830491154168</v>
       </c>
     </row>
     <row r="21" spans="2:25" x14ac:dyDescent="0.3">
@@ -6940,7 +6940,7 @@
       </c>
       <c r="V22" s="26">
         <f>(R23-228195)/228195</f>
-        <v>1124.2351178833105</v>
+        <v>1074.5295795720367</v>
       </c>
     </row>
     <row r="23" spans="2:25" x14ac:dyDescent="0.3">
@@ -6985,7 +6985,7 @@
         <v>114</v>
       </c>
       <c r="R23" s="22">
-        <v>256773027.72538206</v>
+        <v>245430472.41044092</v>
       </c>
       <c r="S23" s="21" t="s">
         <v>128</v>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="V23" s="26">
         <f>(R24-10815)/10815</f>
-        <v>1180.9828008532231</v>
+        <v>1128.5437756346967</v>
       </c>
     </row>
     <row r="24" spans="2:25" x14ac:dyDescent="0.3">
@@ -7040,13 +7040,13 @@
         <v>115</v>
       </c>
       <c r="R24" s="22">
-        <v>12783143.991227608</v>
+        <v>12216015.933489244</v>
       </c>
       <c r="S24" s="21" t="s">
         <v>126</v>
       </c>
       <c r="T24" s="23">
-        <v>287036742.70045835</v>
+        <v>275127059.32777882</v>
       </c>
       <c r="V24" s="8"/>
       <c r="W24" s="8"/>
@@ -7091,7 +7091,7 @@
         <v>242</v>
       </c>
       <c r="T25" s="34">
-        <v>556834253.55156243</v>
+        <v>533014886.80620354</v>
       </c>
       <c r="U25" s="5"/>
       <c r="V25" s="8"/>

</xml_diff>